<commit_message>
feat: Integrasi lengkap data historis Jan-Ags 2026, multi-month neraca, smart expense classification, dan modal laporan bulanan
</commit_message>
<xml_diff>
--- a/file_wisuda_4okt.xlsx
+++ b/file_wisuda_4okt.xlsx
@@ -403,12 +403,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF9900"/>
-        <bgColor rgb="FFFF9900"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF00FF00"/>
         <bgColor rgb="FF00FF00"/>
       </patternFill>
@@ -417,6 +411,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
         <bgColor rgb="FFFF0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF9900"/>
+        <bgColor rgb="FFFF9900"/>
       </patternFill>
     </fill>
   </fills>
@@ -560,7 +560,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="73">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -651,95 +651,92 @@
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="5" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="10" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="11" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="11" fontId="13" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="5" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf borderId="5" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="10" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="10" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="6" fillId="10" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="5" fillId="11" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="5" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="12" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="6" fillId="10" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="10" fontId="15" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="15" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="5" fillId="10" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="7" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="11" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="12" fontId="13" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf borderId="4" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="10" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="8" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="5" fillId="12" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="11" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="11" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="11" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf borderId="5" fillId="12" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="12" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="11" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="11" fontId="15" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="15" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="5" fillId="11" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="7" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="12" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="11" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="8" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="10" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="8" fillId="10" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="8" fillId="12" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -753,13 +750,13 @@
     <xf borderId="10" fillId="0" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="10" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="10" fillId="12" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="10" fillId="10" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="10" fillId="12" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="11" fillId="10" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="11" fillId="12" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="12" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -787,7 +784,7 @@
     <xdr:ext cx="2590800" cy="2590800"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.png" title="Gambar"/>
+        <xdr:cNvPr id="0" name="image1.png" title="Gambar"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -815,7 +812,7 @@
     <xdr:ext cx="209550" cy="142875"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image1.jpg"/>
+        <xdr:cNvPr id="0" name="image2.jpg"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -871,7 +868,7 @@
     <xdr:ext cx="209550" cy="142875"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image4.jpg"/>
+        <xdr:cNvPr id="0" name="image3.jpg"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -927,7 +924,7 @@
     <xdr:ext cx="209550" cy="142875"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.jpg"/>
+        <xdr:cNvPr id="0" name="image4.jpg"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1628,7 +1625,7 @@
       <c r="Q15" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="R15" s="31" t="s">
+      <c r="R15" s="29" t="s">
         <v>19</v>
       </c>
       <c r="S15" s="22">
@@ -1763,22 +1760,22 @@
       <c r="AF17" s="27"/>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="32">
+      <c r="A18" s="31">
         <v>7.0</v>
       </c>
-      <c r="B18" s="33">
+      <c r="B18" s="32">
         <v>0.5</v>
       </c>
-      <c r="C18" s="34" t="s">
+      <c r="C18" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="34" t="s">
+      <c r="D18" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="E18" s="34" t="s">
+      <c r="E18" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="F18" s="34" t="s">
+      <c r="F18" s="33" t="s">
         <v>19</v>
       </c>
       <c r="G18" s="22">
@@ -1825,680 +1822,680 @@
       <c r="AF18" s="27"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="32">
+      <c r="A19" s="31">
         <v>8.0</v>
       </c>
-      <c r="B19" s="33">
+      <c r="B19" s="32">
         <v>0.5208333333333334</v>
       </c>
-      <c r="C19" s="34" t="s">
+      <c r="C19" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="D19" s="34" t="s">
+      <c r="D19" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="E19" s="34" t="s">
+      <c r="E19" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="F19" s="34" t="s">
+      <c r="F19" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="G19" s="35">
+      <c r="G19" s="34">
         <v>8.0</v>
       </c>
-      <c r="H19" s="36">
+      <c r="H19" s="35">
         <v>0.5208333333333334</v>
       </c>
-      <c r="I19" s="35"/>
-      <c r="J19" s="37"/>
-      <c r="K19" s="37"/>
-      <c r="L19" s="37"/>
-      <c r="M19" s="38">
+      <c r="I19" s="34"/>
+      <c r="J19" s="36"/>
+      <c r="K19" s="36"/>
+      <c r="L19" s="36"/>
+      <c r="M19" s="37">
         <v>8.0</v>
       </c>
-      <c r="N19" s="39">
+      <c r="N19" s="38">
         <v>0.5208333333333334</v>
       </c>
-      <c r="O19" s="40" t="s">
+      <c r="O19" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="P19" s="38" t="s">
+      <c r="P19" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="Q19" s="38" t="s">
+      <c r="Q19" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="R19" s="40" t="s">
+      <c r="R19" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="S19" s="32">
+      <c r="S19" s="31">
         <v>8.0</v>
       </c>
-      <c r="T19" s="33">
+      <c r="T19" s="32">
         <v>0.5208333333333334</v>
       </c>
-      <c r="U19" s="41" t="s">
+      <c r="U19" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="V19" s="41" t="s">
+      <c r="V19" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="W19" s="41" t="s">
+      <c r="W19" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="X19" s="41" t="s">
+      <c r="X19" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="Y19" s="38">
+      <c r="Y19" s="37">
         <v>8.0</v>
       </c>
-      <c r="Z19" s="39">
+      <c r="Z19" s="38">
         <v>0.5208333333333334</v>
       </c>
-      <c r="AA19" s="42" t="s">
+      <c r="AA19" s="41" t="s">
         <v>27</v>
       </c>
-      <c r="AB19" s="43" t="s">
+      <c r="AB19" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="AC19" s="43" t="s">
+      <c r="AC19" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="AD19" s="38" t="s">
+      <c r="AD19" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="AE19" s="44"/>
-      <c r="AF19" s="44"/>
+      <c r="AE19" s="43"/>
+      <c r="AF19" s="43"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="32">
+      <c r="A20" s="31">
         <v>9.0</v>
       </c>
-      <c r="B20" s="33">
+      <c r="B20" s="32">
         <v>0.5416666666666666</v>
       </c>
-      <c r="C20" s="34" t="s">
+      <c r="C20" s="33" t="s">
         <v>28</v>
       </c>
-      <c r="D20" s="34" t="s">
+      <c r="D20" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="E20" s="34" t="s">
+      <c r="E20" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="F20" s="34"/>
-      <c r="G20" s="37">
+      <c r="F20" s="33"/>
+      <c r="G20" s="36">
         <v>9.0</v>
       </c>
-      <c r="H20" s="45">
+      <c r="H20" s="44">
         <v>0.5416666666666666</v>
       </c>
-      <c r="I20" s="46"/>
-      <c r="J20" s="46"/>
-      <c r="K20" s="46"/>
-      <c r="L20" s="46"/>
-      <c r="M20" s="32">
+      <c r="I20" s="45"/>
+      <c r="J20" s="45"/>
+      <c r="K20" s="45"/>
+      <c r="L20" s="45"/>
+      <c r="M20" s="31">
         <v>9.0</v>
       </c>
-      <c r="N20" s="33">
+      <c r="N20" s="32">
         <v>0.5416666666666666</v>
       </c>
-      <c r="O20" s="47" t="s">
+      <c r="O20" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="P20" s="48" t="s">
+      <c r="P20" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="Q20" s="48" t="s">
+      <c r="Q20" s="47" t="s">
         <v>23</v>
       </c>
-      <c r="R20" s="34" t="s">
+      <c r="R20" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="S20" s="32">
+      <c r="S20" s="31">
         <v>9.0</v>
       </c>
-      <c r="T20" s="33">
+      <c r="T20" s="32">
         <v>0.5416666666666666</v>
       </c>
-      <c r="U20" s="34" t="s">
+      <c r="U20" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="V20" s="34" t="s">
+      <c r="V20" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="W20" s="34" t="s">
+      <c r="W20" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="X20" s="34" t="s">
+      <c r="X20" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="Y20" s="38">
+      <c r="Y20" s="37">
         <v>9.0</v>
       </c>
-      <c r="Z20" s="39">
+      <c r="Z20" s="38">
         <v>0.5416666666666666</v>
       </c>
-      <c r="AA20" s="42" t="s">
+      <c r="AA20" s="41" t="s">
         <v>31</v>
       </c>
-      <c r="AB20" s="43" t="s">
+      <c r="AB20" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="AC20" s="43" t="s">
+      <c r="AC20" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="AD20" s="49"/>
-      <c r="AE20" s="50"/>
-      <c r="AF20" s="50"/>
+      <c r="AD20" s="48"/>
+      <c r="AE20" s="49"/>
+      <c r="AF20" s="49"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="32">
+      <c r="A21" s="31">
         <v>10.0</v>
       </c>
-      <c r="B21" s="33">
+      <c r="B21" s="32">
         <v>0.5555555555555556</v>
       </c>
-      <c r="C21" s="34" t="s">
+      <c r="C21" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="D21" s="34" t="s">
+      <c r="D21" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="E21" s="34" t="s">
+      <c r="E21" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="F21" s="34" t="s">
+      <c r="F21" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="G21" s="32">
+      <c r="G21" s="31">
         <v>10.0</v>
       </c>
-      <c r="H21" s="33">
+      <c r="H21" s="32">
         <v>0.5555555555555556</v>
       </c>
-      <c r="I21" s="34" t="s">
+      <c r="I21" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="J21" s="34" t="s">
+      <c r="J21" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="K21" s="34" t="s">
+      <c r="K21" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="L21" s="34" t="s">
+      <c r="L21" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="M21" s="32">
+      <c r="M21" s="31">
         <v>10.0</v>
       </c>
-      <c r="N21" s="33">
+      <c r="N21" s="32">
         <v>0.5555555555555556</v>
       </c>
-      <c r="O21" s="51" t="s">
+      <c r="O21" s="50" t="s">
         <v>35</v>
       </c>
-      <c r="P21" s="52" t="s">
+      <c r="P21" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="Q21" s="38" t="s">
+      <c r="Q21" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="R21" s="38" t="s">
+      <c r="R21" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="S21" s="32">
+      <c r="S21" s="31">
         <v>10.0</v>
       </c>
-      <c r="T21" s="33">
+      <c r="T21" s="32">
         <v>0.5555555555555556</v>
       </c>
-      <c r="U21" s="34" t="s">
+      <c r="U21" s="33" t="s">
         <v>37</v>
       </c>
-      <c r="V21" s="34" t="s">
+      <c r="V21" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="W21" s="34" t="s">
+      <c r="W21" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="X21" s="32"/>
-      <c r="Y21" s="32">
+      <c r="X21" s="31"/>
+      <c r="Y21" s="31">
         <v>10.0</v>
       </c>
-      <c r="Z21" s="33">
+      <c r="Z21" s="32">
         <v>0.5555555555555556</v>
       </c>
-      <c r="AA21" s="34" t="s">
+      <c r="AA21" s="33" t="s">
         <v>38</v>
       </c>
-      <c r="AB21" s="34" t="s">
+      <c r="AB21" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="AC21" s="34" t="s">
+      <c r="AC21" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="AD21" s="32"/>
+      <c r="AD21" s="31"/>
       <c r="AE21" s="27"/>
       <c r="AF21" s="27"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="32">
+      <c r="A22" s="31">
         <v>11.0</v>
       </c>
-      <c r="B22" s="33">
+      <c r="B22" s="32">
         <v>0.5694444444444444</v>
       </c>
-      <c r="C22" s="34" t="s">
+      <c r="C22" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="D22" s="34" t="s">
+      <c r="D22" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="E22" s="34" t="s">
+      <c r="E22" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="F22" s="34" t="s">
+      <c r="F22" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="G22" s="37">
+      <c r="G22" s="36">
         <v>11.0</v>
       </c>
-      <c r="H22" s="45">
+      <c r="H22" s="44">
         <v>0.5694444444444444</v>
       </c>
-      <c r="I22" s="37"/>
-      <c r="J22" s="37"/>
-      <c r="K22" s="37"/>
-      <c r="L22" s="37"/>
-      <c r="M22" s="32">
+      <c r="I22" s="36"/>
+      <c r="J22" s="36"/>
+      <c r="K22" s="36"/>
+      <c r="L22" s="36"/>
+      <c r="M22" s="31">
         <v>11.0</v>
       </c>
-      <c r="N22" s="33">
+      <c r="N22" s="32">
         <v>0.5694444444444444</v>
       </c>
-      <c r="O22" s="47" t="s">
+      <c r="O22" s="46" t="s">
         <v>40</v>
       </c>
-      <c r="P22" s="34" t="s">
+      <c r="P22" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="Q22" s="34" t="s">
+      <c r="Q22" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="R22" s="32"/>
-      <c r="S22" s="32">
+      <c r="R22" s="31"/>
+      <c r="S22" s="31">
         <v>11.0</v>
       </c>
-      <c r="T22" s="33">
+      <c r="T22" s="32">
         <v>0.5694444444444444</v>
       </c>
-      <c r="U22" s="34" t="s">
+      <c r="U22" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="V22" s="34" t="s">
+      <c r="V22" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="W22" s="34" t="s">
+      <c r="W22" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="X22" s="34" t="s">
+      <c r="X22" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="Y22" s="32">
+      <c r="Y22" s="31">
         <v>11.0</v>
       </c>
-      <c r="Z22" s="33">
+      <c r="Z22" s="32">
         <v>0.5694444444444444</v>
       </c>
-      <c r="AA22" s="34" t="s">
+      <c r="AA22" s="33" t="s">
         <v>42</v>
       </c>
-      <c r="AB22" s="34" t="s">
+      <c r="AB22" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="AC22" s="34" t="s">
+      <c r="AC22" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="AD22" s="34" t="s">
+      <c r="AD22" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="AE22" s="53"/>
-      <c r="AF22" s="53"/>
+      <c r="AE22" s="52"/>
+      <c r="AF22" s="52"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="38">
+      <c r="A23" s="37">
         <v>13.0</v>
       </c>
-      <c r="B23" s="33">
+      <c r="B23" s="32">
         <v>0.5833333333333334</v>
       </c>
-      <c r="C23" s="38" t="s">
+      <c r="C23" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="D23" s="38" t="s">
+      <c r="D23" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="E23" s="38" t="s">
+      <c r="E23" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="F23" s="38" t="s">
+      <c r="F23" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="G23" s="37">
+      <c r="G23" s="36">
         <v>12.0</v>
       </c>
-      <c r="H23" s="45">
+      <c r="H23" s="44">
         <v>0.5833333333333334</v>
       </c>
-      <c r="I23" s="37"/>
-      <c r="J23" s="54"/>
-      <c r="K23" s="37"/>
-      <c r="L23" s="37"/>
-      <c r="M23" s="32">
+      <c r="I23" s="36"/>
+      <c r="J23" s="53"/>
+      <c r="K23" s="36"/>
+      <c r="L23" s="36"/>
+      <c r="M23" s="31">
         <v>12.0</v>
       </c>
-      <c r="N23" s="33">
+      <c r="N23" s="32">
         <v>0.5833333333333334</v>
       </c>
-      <c r="O23" s="55" t="s">
+      <c r="O23" s="54" t="s">
         <v>44</v>
       </c>
-      <c r="P23" s="38" t="s">
+      <c r="P23" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="Q23" s="38" t="s">
+      <c r="Q23" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="R23" s="38" t="s">
+      <c r="R23" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="S23" s="32">
+      <c r="S23" s="31">
         <v>12.0</v>
       </c>
-      <c r="T23" s="33">
+      <c r="T23" s="32">
         <v>0.5833333333333334</v>
       </c>
-      <c r="U23" s="34" t="s">
+      <c r="U23" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="V23" s="34" t="s">
+      <c r="V23" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="W23" s="34" t="s">
+      <c r="W23" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="X23" s="34" t="s">
+      <c r="X23" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="Y23" s="32">
+      <c r="Y23" s="31">
         <v>12.0</v>
       </c>
-      <c r="Z23" s="33">
+      <c r="Z23" s="32">
         <v>0.5833333333333334</v>
       </c>
-      <c r="AA23" s="38" t="s">
+      <c r="AA23" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="AB23" s="38" t="s">
+      <c r="AB23" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="AC23" s="38" t="s">
+      <c r="AC23" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="AD23" s="51"/>
+      <c r="AD23" s="50"/>
       <c r="AE23" s="27"/>
       <c r="AF23" s="27"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="34">
+      <c r="A24" s="33">
         <v>14.0</v>
       </c>
-      <c r="B24" s="33">
+      <c r="B24" s="32">
         <v>0.5972222222222222</v>
       </c>
-      <c r="C24" s="34" t="s">
+      <c r="C24" s="33" t="s">
         <v>47</v>
       </c>
-      <c r="D24" s="34" t="s">
+      <c r="D24" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="E24" s="34" t="s">
+      <c r="E24" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="F24" s="34" t="s">
+      <c r="F24" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="G24" s="32">
+      <c r="G24" s="31">
         <v>13.0</v>
       </c>
-      <c r="H24" s="33">
+      <c r="H24" s="32">
         <v>0.5972222222222222</v>
       </c>
-      <c r="I24" s="34" t="s">
+      <c r="I24" s="33" t="s">
         <v>48</v>
       </c>
-      <c r="J24" s="34" t="s">
+      <c r="J24" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="K24" s="34" t="s">
+      <c r="K24" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="L24" s="34" t="s">
+      <c r="L24" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="M24" s="32">
+      <c r="M24" s="31">
         <v>13.0</v>
       </c>
-      <c r="N24" s="33">
+      <c r="N24" s="32">
         <v>0.5972222222222222</v>
       </c>
-      <c r="O24" s="38" t="s">
+      <c r="O24" s="37" t="s">
         <v>49</v>
       </c>
-      <c r="P24" s="38" t="s">
+      <c r="P24" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="Q24" s="38" t="s">
+      <c r="Q24" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="R24" s="38" t="s">
+      <c r="R24" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="S24" s="32">
+      <c r="S24" s="31">
         <v>13.0</v>
       </c>
-      <c r="T24" s="33">
+      <c r="T24" s="32">
         <v>0.5972222222222222</v>
       </c>
-      <c r="U24" s="34" t="s">
+      <c r="U24" s="33" t="s">
         <v>50</v>
       </c>
-      <c r="V24" s="34" t="s">
+      <c r="V24" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="W24" s="34" t="s">
+      <c r="W24" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="X24" s="34" t="s">
+      <c r="X24" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="Y24" s="37">
+      <c r="Y24" s="36">
         <v>13.0</v>
       </c>
-      <c r="Z24" s="45">
+      <c r="Z24" s="44">
         <v>0.5972222222222222</v>
       </c>
-      <c r="AA24" s="37"/>
-      <c r="AB24" s="37"/>
-      <c r="AC24" s="37"/>
-      <c r="AD24" s="37"/>
+      <c r="AA24" s="36"/>
+      <c r="AB24" s="36"/>
+      <c r="AC24" s="36"/>
+      <c r="AD24" s="36"/>
       <c r="AE24" s="27"/>
       <c r="AF24" s="27"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="37">
+      <c r="A25" s="36">
         <v>14.0</v>
       </c>
-      <c r="B25" s="45">
+      <c r="B25" s="44">
         <v>0.6111111111111112</v>
       </c>
-      <c r="C25" s="37"/>
-      <c r="D25" s="37"/>
-      <c r="E25" s="37"/>
-      <c r="F25" s="37"/>
-      <c r="G25" s="32">
+      <c r="C25" s="36"/>
+      <c r="D25" s="36"/>
+      <c r="E25" s="36"/>
+      <c r="F25" s="36"/>
+      <c r="G25" s="31">
         <v>14.0</v>
       </c>
-      <c r="H25" s="33">
+      <c r="H25" s="32">
         <v>0.6111111111111112</v>
       </c>
-      <c r="I25" s="34" t="s">
+      <c r="I25" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="J25" s="34" t="s">
+      <c r="J25" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="K25" s="34" t="s">
+      <c r="K25" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="L25" s="34" t="s">
+      <c r="L25" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="M25" s="32">
+      <c r="M25" s="31">
         <v>14.0</v>
       </c>
-      <c r="N25" s="33">
+      <c r="N25" s="32">
         <v>0.6111111111111112</v>
       </c>
-      <c r="O25" s="34" t="s">
+      <c r="O25" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="P25" s="34" t="s">
+      <c r="P25" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="Q25" s="34" t="s">
+      <c r="Q25" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="R25" s="32"/>
-      <c r="S25" s="32">
+      <c r="R25" s="31"/>
+      <c r="S25" s="31">
         <v>14.0</v>
       </c>
-      <c r="T25" s="33">
+      <c r="T25" s="32">
         <v>0.6111111111111112</v>
       </c>
-      <c r="U25" s="34" t="s">
+      <c r="U25" s="33" t="s">
         <v>53</v>
       </c>
-      <c r="V25" s="34" t="s">
+      <c r="V25" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="W25" s="34" t="s">
+      <c r="W25" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="X25" s="34" t="s">
+      <c r="X25" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="Y25" s="32">
+      <c r="Y25" s="31">
         <v>14.0</v>
       </c>
-      <c r="Z25" s="33">
+      <c r="Z25" s="32">
         <v>0.6111111111111112</v>
       </c>
-      <c r="AA25" s="34" t="s">
+      <c r="AA25" s="33" t="s">
         <v>54</v>
       </c>
-      <c r="AB25" s="34" t="s">
+      <c r="AB25" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="AC25" s="34" t="s">
+      <c r="AC25" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="AD25" s="34" t="s">
+      <c r="AD25" s="33" t="s">
         <v>19</v>
       </c>
       <c r="AE25" s="27"/>
       <c r="AF25" s="27"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="37">
+      <c r="A26" s="36">
         <v>15.0</v>
       </c>
-      <c r="B26" s="45">
+      <c r="B26" s="44">
         <v>0.625</v>
       </c>
-      <c r="C26" s="46"/>
-      <c r="D26" s="46"/>
-      <c r="E26" s="46"/>
-      <c r="F26" s="37"/>
-      <c r="G26" s="32">
+      <c r="C26" s="45"/>
+      <c r="D26" s="45"/>
+      <c r="E26" s="45"/>
+      <c r="F26" s="36"/>
+      <c r="G26" s="31">
         <v>15.0</v>
       </c>
-      <c r="H26" s="33">
+      <c r="H26" s="32">
         <v>0.625</v>
       </c>
-      <c r="I26" s="34" t="s">
+      <c r="I26" s="33" t="s">
         <v>55</v>
       </c>
-      <c r="J26" s="34" t="s">
+      <c r="J26" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="K26" s="34" t="s">
+      <c r="K26" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="L26" s="34" t="s">
+      <c r="L26" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="M26" s="32">
+      <c r="M26" s="31">
         <v>15.0</v>
       </c>
-      <c r="N26" s="33">
+      <c r="N26" s="32">
         <v>0.625</v>
       </c>
-      <c r="O26" s="34" t="s">
+      <c r="O26" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="P26" s="34" t="s">
+      <c r="P26" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="Q26" s="34" t="s">
+      <c r="Q26" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="R26" s="32"/>
-      <c r="S26" s="32">
+      <c r="R26" s="31"/>
+      <c r="S26" s="31">
         <v>15.0</v>
       </c>
-      <c r="T26" s="33">
+      <c r="T26" s="32">
         <v>0.625</v>
       </c>
-      <c r="U26" s="34" t="s">
+      <c r="U26" s="33" t="s">
         <v>57</v>
       </c>
-      <c r="V26" s="34" t="s">
+      <c r="V26" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="W26" s="34" t="s">
+      <c r="W26" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="X26" s="34" t="s">
+      <c r="X26" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="Y26" s="32">
+      <c r="Y26" s="31">
         <v>15.0</v>
       </c>
-      <c r="Z26" s="33">
+      <c r="Z26" s="32">
         <v>0.625</v>
       </c>
-      <c r="AA26" s="34" t="s">
+      <c r="AA26" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="AB26" s="34" t="s">
+      <c r="AB26" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="AC26" s="34" t="s">
+      <c r="AC26" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="AD26" s="34" t="s">
+      <c r="AD26" s="33" t="s">
         <v>59</v>
       </c>
       <c r="AE26" s="27"/>
@@ -2515,296 +2512,296 @@
       <c r="D27" s="28"/>
       <c r="E27" s="28"/>
       <c r="F27" s="28"/>
-      <c r="G27" s="32">
+      <c r="G27" s="31">
         <v>16.0</v>
       </c>
-      <c r="H27" s="33">
+      <c r="H27" s="32">
         <v>0.6388888888888888</v>
       </c>
-      <c r="I27" s="34" t="s">
+      <c r="I27" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="J27" s="34" t="s">
+      <c r="J27" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="K27" s="34" t="s">
+      <c r="K27" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="L27" s="34" t="s">
+      <c r="L27" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="M27" s="32">
+      <c r="M27" s="31">
         <v>16.0</v>
       </c>
-      <c r="N27" s="33">
+      <c r="N27" s="32">
         <v>0.6388888888888888</v>
       </c>
-      <c r="O27" s="34" t="s">
+      <c r="O27" s="33" t="s">
         <v>62</v>
       </c>
-      <c r="P27" s="34" t="s">
+      <c r="P27" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="Q27" s="34" t="s">
+      <c r="Q27" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="R27" s="34" t="s">
+      <c r="R27" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="S27" s="37">
+      <c r="S27" s="36">
         <v>16.0</v>
       </c>
-      <c r="T27" s="45">
+      <c r="T27" s="44">
         <v>0.6388888888888888</v>
       </c>
-      <c r="U27" s="37"/>
-      <c r="V27" s="37"/>
-      <c r="W27" s="37"/>
-      <c r="X27" s="37"/>
-      <c r="Y27" s="32">
+      <c r="U27" s="36"/>
+      <c r="V27" s="36"/>
+      <c r="W27" s="36"/>
+      <c r="X27" s="36"/>
+      <c r="Y27" s="31">
         <v>16.0</v>
       </c>
-      <c r="Z27" s="33">
+      <c r="Z27" s="32">
         <v>0.6388888888888888</v>
       </c>
-      <c r="AA27" s="34" t="s">
+      <c r="AA27" s="33" t="s">
         <v>63</v>
       </c>
-      <c r="AB27" s="34" t="s">
+      <c r="AB27" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="AC27" s="34" t="s">
+      <c r="AC27" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="AD27" s="34" t="s">
+      <c r="AD27" s="33" t="s">
         <v>19</v>
       </c>
       <c r="AE27" s="27"/>
       <c r="AF27" s="27"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="32">
+      <c r="A28" s="31">
         <v>17.0</v>
       </c>
-      <c r="B28" s="33">
+      <c r="B28" s="32">
         <v>0.6527777777777778</v>
       </c>
-      <c r="C28" s="34" t="s">
+      <c r="C28" s="33" t="s">
         <v>64</v>
       </c>
-      <c r="D28" s="34" t="s">
+      <c r="D28" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="E28" s="34" t="s">
+      <c r="E28" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="F28" s="34" t="s">
+      <c r="F28" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="G28" s="32">
+      <c r="G28" s="31">
         <v>17.0</v>
       </c>
-      <c r="H28" s="33">
+      <c r="H28" s="32">
         <v>0.6527777777777778</v>
       </c>
-      <c r="I28" s="34" t="s">
+      <c r="I28" s="33" t="s">
         <v>65</v>
       </c>
-      <c r="J28" s="34" t="s">
+      <c r="J28" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="K28" s="34" t="s">
+      <c r="K28" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="L28" s="34" t="s">
+      <c r="L28" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="M28" s="32">
+      <c r="M28" s="31">
         <v>17.0</v>
       </c>
-      <c r="N28" s="33">
+      <c r="N28" s="32">
         <v>0.6527777777777778</v>
       </c>
-      <c r="O28" s="38" t="s">
+      <c r="O28" s="37" t="s">
         <v>66</v>
       </c>
-      <c r="P28" s="38" t="s">
+      <c r="P28" s="37" t="s">
         <v>67</v>
       </c>
-      <c r="Q28" s="38" t="s">
+      <c r="Q28" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="R28" s="56" t="s">
+      <c r="R28" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="S28" s="37">
+      <c r="S28" s="36">
         <v>17.0</v>
       </c>
-      <c r="T28" s="45">
+      <c r="T28" s="44">
         <v>0.6527777777777778</v>
       </c>
-      <c r="U28" s="37"/>
-      <c r="V28" s="37"/>
-      <c r="W28" s="37"/>
-      <c r="X28" s="37"/>
-      <c r="Y28" s="32">
+      <c r="U28" s="36"/>
+      <c r="V28" s="36"/>
+      <c r="W28" s="36"/>
+      <c r="X28" s="36"/>
+      <c r="Y28" s="31">
         <v>17.0</v>
       </c>
-      <c r="Z28" s="33">
+      <c r="Z28" s="32">
         <v>0.6527777777777778</v>
       </c>
-      <c r="AA28" s="34" t="s">
+      <c r="AA28" s="33" t="s">
         <v>68</v>
       </c>
-      <c r="AB28" s="34" t="s">
+      <c r="AB28" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="AC28" s="34" t="s">
+      <c r="AC28" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="AD28" s="34" t="s">
+      <c r="AD28" s="33" t="s">
         <v>19</v>
       </c>
       <c r="AE28" s="27"/>
       <c r="AF28" s="27"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="32">
+      <c r="A29" s="31">
         <v>18.0</v>
       </c>
-      <c r="B29" s="33">
+      <c r="B29" s="32">
         <v>0.6666666666666666</v>
       </c>
-      <c r="C29" s="34" t="s">
+      <c r="C29" s="33" t="s">
         <v>69</v>
       </c>
-      <c r="D29" s="34" t="s">
+      <c r="D29" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="E29" s="34" t="s">
+      <c r="E29" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="F29" s="34" t="s">
+      <c r="F29" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="G29" s="37">
+      <c r="G29" s="36">
         <v>18.0</v>
       </c>
-      <c r="H29" s="45">
+      <c r="H29" s="44">
         <v>0.6666666666666666</v>
       </c>
-      <c r="I29" s="37"/>
-      <c r="J29" s="37"/>
-      <c r="K29" s="37"/>
-      <c r="L29" s="37"/>
-      <c r="M29" s="32">
+      <c r="I29" s="36"/>
+      <c r="J29" s="36"/>
+      <c r="K29" s="36"/>
+      <c r="L29" s="36"/>
+      <c r="M29" s="31">
         <v>18.0</v>
       </c>
-      <c r="N29" s="33">
+      <c r="N29" s="32">
         <v>0.6666666666666666</v>
       </c>
-      <c r="O29" s="34" t="s">
+      <c r="O29" s="33" t="s">
         <v>70</v>
       </c>
-      <c r="P29" s="34" t="s">
+      <c r="P29" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="Q29" s="34" t="s">
+      <c r="Q29" s="33" t="s">
         <v>71</v>
       </c>
-      <c r="R29" s="34" t="s">
+      <c r="R29" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="S29" s="38">
+      <c r="S29" s="37">
         <v>18.0</v>
       </c>
-      <c r="T29" s="39">
+      <c r="T29" s="38">
         <v>0.6666666666666666</v>
       </c>
-      <c r="U29" s="48" t="s">
+      <c r="U29" s="47" t="s">
         <v>72</v>
       </c>
-      <c r="V29" s="48" t="s">
+      <c r="V29" s="47" t="s">
         <v>67</v>
       </c>
-      <c r="W29" s="48" t="s">
+      <c r="W29" s="47" t="s">
         <v>23</v>
       </c>
-      <c r="X29" s="56" t="s">
+      <c r="X29" s="55" t="s">
         <v>19</v>
       </c>
-      <c r="Y29" s="32">
+      <c r="Y29" s="31">
         <v>18.0</v>
       </c>
-      <c r="Z29" s="33">
+      <c r="Z29" s="32">
         <v>0.6666666666666666</v>
       </c>
-      <c r="AA29" s="48" t="s">
+      <c r="AA29" s="47" t="s">
         <v>73</v>
       </c>
-      <c r="AB29" s="48" t="s">
+      <c r="AB29" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="AC29" s="48" t="s">
+      <c r="AC29" s="47" t="s">
         <v>23</v>
       </c>
-      <c r="AD29" s="57" t="s">
+      <c r="AD29" s="56" t="s">
         <v>19</v>
       </c>
-      <c r="AE29" s="58"/>
-      <c r="AF29" s="59"/>
+      <c r="AE29" s="57"/>
+      <c r="AF29" s="58"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="32">
+      <c r="A30" s="31">
         <v>19.0</v>
       </c>
-      <c r="B30" s="33">
+      <c r="B30" s="32">
         <v>0.6805555555555556</v>
       </c>
-      <c r="C30" s="34" t="s">
+      <c r="C30" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="D30" s="34" t="s">
+      <c r="D30" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="E30" s="34" t="s">
+      <c r="E30" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="F30" s="32"/>
-      <c r="G30" s="32">
+      <c r="F30" s="31"/>
+      <c r="G30" s="31">
         <v>19.0</v>
       </c>
-      <c r="H30" s="33">
+      <c r="H30" s="32">
         <v>0.6805555555555556</v>
       </c>
-      <c r="I30" s="34" t="s">
+      <c r="I30" s="33" t="s">
         <v>75</v>
       </c>
-      <c r="J30" s="34" t="s">
+      <c r="J30" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="K30" s="34" t="s">
+      <c r="K30" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="L30" s="34" t="s">
+      <c r="L30" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="M30" s="32">
+      <c r="M30" s="31">
         <v>19.0</v>
       </c>
-      <c r="N30" s="33">
+      <c r="N30" s="32">
         <v>0.6805555555555556</v>
       </c>
-      <c r="O30" s="34" t="s">
+      <c r="O30" s="33" t="s">
         <v>76</v>
       </c>
-      <c r="P30" s="34" t="s">
+      <c r="P30" s="33" t="s">
         <v>67</v>
       </c>
-      <c r="Q30" s="34" t="s">
+      <c r="Q30" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="R30" s="34" t="s">
+      <c r="R30" s="33" t="s">
         <v>59</v>
       </c>
       <c r="S30" s="22">
@@ -2831,22 +2828,22 @@
       <c r="AF30" s="27"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="32">
+      <c r="A31" s="31">
         <v>20.0</v>
       </c>
-      <c r="B31" s="33">
+      <c r="B31" s="32">
         <v>0.6944444444444444</v>
       </c>
-      <c r="C31" s="34" t="s">
+      <c r="C31" s="33" t="s">
         <v>77</v>
       </c>
-      <c r="D31" s="34" t="s">
+      <c r="D31" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="E31" s="34" t="s">
+      <c r="E31" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="F31" s="34" t="s">
+      <c r="F31" s="33" t="s">
         <v>16</v>
       </c>
       <c r="G31" s="22">
@@ -2859,18 +2856,18 @@
       <c r="J31" s="22"/>
       <c r="K31" s="22"/>
       <c r="L31" s="22"/>
-      <c r="M31" s="60">
+      <c r="M31" s="59">
         <v>20.0</v>
       </c>
-      <c r="N31" s="61">
+      <c r="N31" s="60">
         <v>0.6944444444444444</v>
       </c>
-      <c r="O31" s="62" t="s">
+      <c r="O31" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="P31" s="63"/>
-      <c r="Q31" s="63"/>
-      <c r="R31" s="64"/>
+      <c r="P31" s="62"/>
+      <c r="Q31" s="62"/>
+      <c r="R31" s="63"/>
       <c r="S31" s="22">
         <v>20.0</v>
       </c>
@@ -2915,18 +2912,18 @@
       <c r="J32" s="22"/>
       <c r="K32" s="22"/>
       <c r="L32" s="22"/>
-      <c r="M32" s="60">
+      <c r="M32" s="59">
         <v>21.0</v>
       </c>
-      <c r="N32" s="61">
+      <c r="N32" s="60">
         <v>0.7083333333333334</v>
       </c>
-      <c r="O32" s="62" t="s">
+      <c r="O32" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="P32" s="63"/>
-      <c r="Q32" s="63"/>
-      <c r="R32" s="64"/>
+      <c r="P32" s="62"/>
+      <c r="Q32" s="62"/>
+      <c r="R32" s="63"/>
       <c r="S32" s="22">
         <v>21.0</v>
       </c>
@@ -2971,18 +2968,18 @@
       <c r="J33" s="22"/>
       <c r="K33" s="22"/>
       <c r="L33" s="22"/>
-      <c r="M33" s="60">
+      <c r="M33" s="59">
         <v>22.0</v>
       </c>
-      <c r="N33" s="61">
+      <c r="N33" s="60">
         <v>0.7222222222222222</v>
       </c>
-      <c r="O33" s="62" t="s">
+      <c r="O33" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="P33" s="63"/>
-      <c r="Q33" s="63"/>
-      <c r="R33" s="64"/>
+      <c r="P33" s="62"/>
+      <c r="Q33" s="62"/>
+      <c r="R33" s="63"/>
       <c r="S33" s="22">
         <v>22.0</v>
       </c>
@@ -3029,18 +3026,18 @@
       <c r="J34" s="22"/>
       <c r="K34" s="22"/>
       <c r="L34" s="22"/>
-      <c r="M34" s="60">
+      <c r="M34" s="59">
         <v>23.0</v>
       </c>
-      <c r="N34" s="61">
+      <c r="N34" s="60">
         <v>0.7361111111111112</v>
       </c>
-      <c r="O34" s="62" t="s">
+      <c r="O34" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="P34" s="63"/>
-      <c r="Q34" s="63"/>
-      <c r="R34" s="64"/>
+      <c r="P34" s="62"/>
+      <c r="Q34" s="62"/>
+      <c r="R34" s="63"/>
       <c r="S34" s="22">
         <v>23.0</v>
       </c>
@@ -3085,18 +3082,18 @@
       <c r="J35" s="22"/>
       <c r="K35" s="22"/>
       <c r="L35" s="22"/>
-      <c r="M35" s="60">
+      <c r="M35" s="59">
         <v>24.0</v>
       </c>
-      <c r="N35" s="61">
+      <c r="N35" s="60">
         <v>0.75</v>
       </c>
-      <c r="O35" s="62" t="s">
+      <c r="O35" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="P35" s="63"/>
-      <c r="Q35" s="63"/>
-      <c r="R35" s="64"/>
+      <c r="P35" s="62"/>
+      <c r="Q35" s="62"/>
+      <c r="R35" s="63"/>
       <c r="S35" s="22">
         <v>24.0</v>
       </c>
@@ -3141,18 +3138,18 @@
       <c r="J36" s="22"/>
       <c r="K36" s="22"/>
       <c r="L36" s="22"/>
-      <c r="M36" s="60">
+      <c r="M36" s="59">
         <v>25.0</v>
       </c>
-      <c r="N36" s="61">
+      <c r="N36" s="60">
         <v>0.7638888888888888</v>
       </c>
-      <c r="O36" s="62" t="s">
+      <c r="O36" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="P36" s="63"/>
-      <c r="Q36" s="63"/>
-      <c r="R36" s="64"/>
+      <c r="P36" s="62"/>
+      <c r="Q36" s="62"/>
+      <c r="R36" s="63"/>
       <c r="S36" s="22">
         <v>25.0</v>
       </c>
@@ -3197,18 +3194,18 @@
       <c r="J37" s="22"/>
       <c r="K37" s="22"/>
       <c r="L37" s="22"/>
-      <c r="M37" s="60">
+      <c r="M37" s="59">
         <v>26.0</v>
       </c>
-      <c r="N37" s="61">
+      <c r="N37" s="60">
         <v>0.7777777777777778</v>
       </c>
-      <c r="O37" s="62" t="s">
+      <c r="O37" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="P37" s="63"/>
-      <c r="Q37" s="63"/>
-      <c r="R37" s="64"/>
+      <c r="P37" s="62"/>
+      <c r="Q37" s="62"/>
+      <c r="R37" s="63"/>
       <c r="S37" s="22">
         <v>26.0</v>
       </c>
@@ -3253,18 +3250,18 @@
       <c r="J38" s="22"/>
       <c r="K38" s="22"/>
       <c r="L38" s="22"/>
-      <c r="M38" s="60">
+      <c r="M38" s="59">
         <v>27.0</v>
       </c>
-      <c r="N38" s="61">
+      <c r="N38" s="60">
         <v>0.7916666666666666</v>
       </c>
-      <c r="O38" s="62" t="s">
+      <c r="O38" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="P38" s="63"/>
-      <c r="Q38" s="63"/>
-      <c r="R38" s="64"/>
+      <c r="P38" s="62"/>
+      <c r="Q38" s="62"/>
+      <c r="R38" s="63"/>
       <c r="S38" s="22">
         <v>27.0</v>
       </c>
@@ -3309,18 +3306,18 @@
       <c r="J39" s="22"/>
       <c r="K39" s="22"/>
       <c r="L39" s="22"/>
-      <c r="M39" s="60">
+      <c r="M39" s="59">
         <v>28.0</v>
       </c>
-      <c r="N39" s="61">
+      <c r="N39" s="60">
         <v>0.8055555555555556</v>
       </c>
-      <c r="O39" s="62" t="s">
+      <c r="O39" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="P39" s="63"/>
-      <c r="Q39" s="63"/>
-      <c r="R39" s="64"/>
+      <c r="P39" s="62"/>
+      <c r="Q39" s="62"/>
+      <c r="R39" s="63"/>
       <c r="S39" s="22">
         <v>28.0</v>
       </c>
@@ -3340,7 +3337,7 @@
       <c r="AA39" s="22"/>
       <c r="AB39" s="22"/>
       <c r="AC39" s="22"/>
-      <c r="AD39" s="65"/>
+      <c r="AD39" s="64"/>
       <c r="AE39" s="1"/>
       <c r="AF39" s="1"/>
     </row>
@@ -3365,18 +3362,18 @@
       <c r="J40" s="22"/>
       <c r="K40" s="22"/>
       <c r="L40" s="22"/>
-      <c r="M40" s="60">
+      <c r="M40" s="59">
         <v>29.0</v>
       </c>
-      <c r="N40" s="61">
+      <c r="N40" s="60">
         <v>0.8194444444444444</v>
       </c>
-      <c r="O40" s="62" t="s">
+      <c r="O40" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="P40" s="63"/>
-      <c r="Q40" s="63"/>
-      <c r="R40" s="64"/>
+      <c r="P40" s="62"/>
+      <c r="Q40" s="62"/>
+      <c r="R40" s="63"/>
       <c r="S40" s="22">
         <v>29.0</v>
       </c>
@@ -3396,7 +3393,7 @@
       <c r="AA40" s="22"/>
       <c r="AB40" s="22"/>
       <c r="AC40" s="22"/>
-      <c r="AD40" s="65"/>
+      <c r="AD40" s="64"/>
       <c r="AE40" s="1"/>
       <c r="AF40" s="1"/>
     </row>
@@ -3421,18 +3418,18 @@
       <c r="J41" s="22"/>
       <c r="K41" s="22"/>
       <c r="L41" s="22"/>
-      <c r="M41" s="60">
+      <c r="M41" s="59">
         <v>30.0</v>
       </c>
-      <c r="N41" s="61">
+      <c r="N41" s="60">
         <v>0.8333333333333334</v>
       </c>
-      <c r="O41" s="62" t="s">
+      <c r="O41" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="P41" s="63"/>
-      <c r="Q41" s="63"/>
-      <c r="R41" s="64"/>
+      <c r="P41" s="62"/>
+      <c r="Q41" s="62"/>
+      <c r="R41" s="63"/>
       <c r="S41" s="22">
         <v>30.0</v>
       </c>
@@ -3452,7 +3449,7 @@
       <c r="AA41" s="22"/>
       <c r="AB41" s="22"/>
       <c r="AC41" s="22"/>
-      <c r="AD41" s="65"/>
+      <c r="AD41" s="64"/>
       <c r="AE41" s="1"/>
       <c r="AF41" s="1"/>
     </row>
@@ -3477,18 +3474,18 @@
       <c r="J42" s="22"/>
       <c r="K42" s="22"/>
       <c r="L42" s="22"/>
-      <c r="M42" s="60">
+      <c r="M42" s="59">
         <v>31.0</v>
       </c>
-      <c r="N42" s="61">
+      <c r="N42" s="60">
         <v>0.8472222222222222</v>
       </c>
-      <c r="O42" s="62" t="s">
+      <c r="O42" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="P42" s="63"/>
-      <c r="Q42" s="63"/>
-      <c r="R42" s="64"/>
+      <c r="P42" s="62"/>
+      <c r="Q42" s="62"/>
+      <c r="R42" s="63"/>
       <c r="S42" s="22">
         <v>31.0</v>
       </c>
@@ -3508,63 +3505,63 @@
       <c r="AA42" s="22"/>
       <c r="AB42" s="22"/>
       <c r="AC42" s="22"/>
-      <c r="AD42" s="65"/>
+      <c r="AD42" s="64"/>
       <c r="AE42" s="1"/>
       <c r="AF42" s="1"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="66">
+      <c r="A43" s="65">
         <v>32.0</v>
       </c>
-      <c r="B43" s="67">
+      <c r="B43" s="66">
         <v>0.8611111111111112</v>
       </c>
-      <c r="C43" s="66"/>
-      <c r="D43" s="66"/>
-      <c r="E43" s="66"/>
-      <c r="F43" s="66"/>
-      <c r="G43" s="66">
+      <c r="C43" s="65"/>
+      <c r="D43" s="65"/>
+      <c r="E43" s="65"/>
+      <c r="F43" s="65"/>
+      <c r="G43" s="65">
         <v>32.0</v>
       </c>
-      <c r="H43" s="67">
+      <c r="H43" s="66">
         <v>0.8611111111111112</v>
       </c>
-      <c r="I43" s="66"/>
-      <c r="J43" s="66"/>
-      <c r="K43" s="66"/>
-      <c r="L43" s="66"/>
-      <c r="M43" s="68">
+      <c r="I43" s="65"/>
+      <c r="J43" s="65"/>
+      <c r="K43" s="65"/>
+      <c r="L43" s="65"/>
+      <c r="M43" s="67">
         <v>32.0</v>
       </c>
-      <c r="N43" s="69">
+      <c r="N43" s="68">
         <v>0.8611111111111112</v>
       </c>
-      <c r="O43" s="70" t="s">
+      <c r="O43" s="69" t="s">
         <v>78</v>
       </c>
-      <c r="P43" s="71"/>
-      <c r="Q43" s="71"/>
-      <c r="R43" s="72"/>
-      <c r="S43" s="66">
+      <c r="P43" s="70"/>
+      <c r="Q43" s="70"/>
+      <c r="R43" s="71"/>
+      <c r="S43" s="65">
         <v>32.0</v>
       </c>
-      <c r="T43" s="67">
+      <c r="T43" s="66">
         <v>0.8611111111111112</v>
       </c>
-      <c r="U43" s="66"/>
-      <c r="V43" s="66"/>
-      <c r="W43" s="66"/>
-      <c r="X43" s="66"/>
-      <c r="Y43" s="66">
+      <c r="U43" s="65"/>
+      <c r="V43" s="65"/>
+      <c r="W43" s="65"/>
+      <c r="X43" s="65"/>
+      <c r="Y43" s="65">
         <v>32.0</v>
       </c>
-      <c r="Z43" s="67">
+      <c r="Z43" s="66">
         <v>0.8611111111111112</v>
       </c>
-      <c r="AA43" s="66"/>
-      <c r="AB43" s="66"/>
-      <c r="AC43" s="66"/>
-      <c r="AD43" s="73"/>
+      <c r="AA43" s="65"/>
+      <c r="AB43" s="65"/>
+      <c r="AC43" s="65"/>
+      <c r="AD43" s="72"/>
       <c r="AE43" s="1"/>
       <c r="AF43" s="1"/>
     </row>

</xml_diff>

<commit_message>
feat(history): buka penuh dashboard Jan-Ags 2026, multi-month switcher, dan cache instan
</commit_message>
<xml_diff>
--- a/file_wisuda_4okt.xlsx
+++ b/file_wisuda_4okt.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="81">
   <si>
     <t xml:space="preserve">Graduation Schedule 
 </t>
@@ -85,6 +85,9 @@
     <t>Graduation</t>
   </si>
   <si>
+    <t>Yeni A</t>
+  </si>
+  <si>
     <t>Nurul Indah Amalia</t>
   </si>
   <si>
@@ -115,7 +118,7 @@
     <t>Azhar</t>
   </si>
   <si>
-    <t>Yeni A</t>
+    <t xml:space="preserve"> </t>
   </si>
   <si>
     <t>Fedinda Nara</t>
@@ -199,6 +202,9 @@
     <t>dp 200</t>
   </si>
   <si>
+    <t>Ridho</t>
+  </si>
+  <si>
     <t>Indriyani</t>
   </si>
   <si>
@@ -254,9 +260,6 @@
   </si>
   <si>
     <t>CLOSED</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -671,9 +674,6 @@
     <xf borderId="5" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="10" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf borderId="5" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
@@ -720,6 +720,9 @@
     </xf>
     <xf borderId="5" fillId="10" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="5" fillId="10" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="8" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
@@ -896,7 +899,7 @@
     <xdr:ext cx="209550" cy="142875"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image5.jpg"/>
+        <xdr:cNvPr id="0" name="image4.jpg"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -924,7 +927,7 @@
     <xdr:ext cx="209550" cy="142875"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image4.jpg"/>
+        <xdr:cNvPr id="0" name="image5.jpg"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1706,16 +1709,24 @@
       <c r="AF16" s="27"/>
     </row>
     <row r="17" ht="15.75" customHeight="1">
-      <c r="A17" s="22">
+      <c r="A17" s="24">
         <v>6.0</v>
       </c>
-      <c r="B17" s="23">
+      <c r="B17" s="25">
         <v>0.4791666666666667</v>
       </c>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22"/>
+      <c r="C17" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="D17" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="E17" s="26" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" s="26" t="s">
+        <v>19</v>
+      </c>
       <c r="G17" s="22">
         <v>6.0</v>
       </c>
@@ -1767,13 +1778,13 @@
         <v>0.5</v>
       </c>
       <c r="C18" s="33" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D18" s="33" t="s">
         <v>21</v>
       </c>
       <c r="E18" s="33" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F18" s="33" t="s">
         <v>19</v>
@@ -1822,20 +1833,20 @@
       <c r="AF18" s="27"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="31">
+      <c r="A19" s="24">
         <v>8.0</v>
       </c>
-      <c r="B19" s="32">
+      <c r="B19" s="25">
         <v>0.5208333333333334</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D19" s="33" t="s">
         <v>21</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F19" s="33" t="s">
         <v>19</v>
@@ -1850,62 +1861,62 @@
       <c r="J19" s="36"/>
       <c r="K19" s="36"/>
       <c r="L19" s="36"/>
-      <c r="M19" s="37">
+      <c r="M19" s="29">
         <v>8.0</v>
       </c>
-      <c r="N19" s="38">
+      <c r="N19" s="30">
         <v>0.5208333333333334</v>
       </c>
-      <c r="O19" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="P19" s="37" t="s">
+      <c r="O19" s="37" t="s">
+        <v>26</v>
+      </c>
+      <c r="P19" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="Q19" s="37" t="s">
+      <c r="Q19" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="R19" s="39" t="s">
+      <c r="R19" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="S19" s="31">
+      <c r="S19" s="24">
         <v>8.0</v>
       </c>
-      <c r="T19" s="32">
+      <c r="T19" s="25">
         <v>0.5208333333333334</v>
       </c>
-      <c r="U19" s="40" t="s">
-        <v>26</v>
-      </c>
-      <c r="V19" s="40" t="s">
+      <c r="U19" s="39" t="s">
+        <v>27</v>
+      </c>
+      <c r="V19" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="W19" s="40" t="s">
-        <v>23</v>
-      </c>
-      <c r="X19" s="40" t="s">
+      <c r="W19" s="39" t="s">
+        <v>24</v>
+      </c>
+      <c r="X19" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="Y19" s="37">
+      <c r="Y19" s="29">
         <v>8.0</v>
       </c>
-      <c r="Z19" s="38">
+      <c r="Z19" s="30">
         <v>0.5208333333333334</v>
       </c>
-      <c r="AA19" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB19" s="42" t="s">
+      <c r="AA19" s="40" t="s">
+        <v>28</v>
+      </c>
+      <c r="AB19" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="AC19" s="42" t="s">
+      <c r="AC19" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="AD19" s="37" t="s">
+      <c r="AD19" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="AE19" s="43"/>
-      <c r="AF19" s="43"/>
+      <c r="AE19" s="42"/>
+      <c r="AF19" s="42"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="31">
@@ -1915,39 +1926,39 @@
         <v>0.5416666666666666</v>
       </c>
       <c r="C20" s="33" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D20" s="33" t="s">
         <v>21</v>
       </c>
       <c r="E20" s="33" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F20" s="33"/>
       <c r="G20" s="36">
         <v>9.0</v>
       </c>
-      <c r="H20" s="44">
+      <c r="H20" s="43">
         <v>0.5416666666666666</v>
       </c>
-      <c r="I20" s="45"/>
-      <c r="J20" s="45"/>
-      <c r="K20" s="45"/>
-      <c r="L20" s="45"/>
+      <c r="I20" s="44"/>
+      <c r="J20" s="44"/>
+      <c r="K20" s="44"/>
+      <c r="L20" s="44"/>
       <c r="M20" s="31">
         <v>9.0</v>
       </c>
       <c r="N20" s="32">
         <v>0.5416666666666666</v>
       </c>
-      <c r="O20" s="46" t="s">
-        <v>29</v>
-      </c>
-      <c r="P20" s="47" t="s">
+      <c r="O20" s="45" t="s">
+        <v>30</v>
+      </c>
+      <c r="P20" s="46" t="s">
         <v>21</v>
       </c>
-      <c r="Q20" s="47" t="s">
-        <v>23</v>
+      <c r="Q20" s="46" t="s">
+        <v>24</v>
       </c>
       <c r="R20" s="33" t="s">
         <v>19</v>
@@ -1959,55 +1970,49 @@
         <v>0.5416666666666666</v>
       </c>
       <c r="U20" s="33" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="V20" s="33" t="s">
         <v>21</v>
       </c>
       <c r="W20" s="33" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="X20" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="Y20" s="37">
+      <c r="Y20" s="29">
         <v>9.0</v>
       </c>
-      <c r="Z20" s="38">
+      <c r="Z20" s="30">
         <v>0.5416666666666666</v>
       </c>
-      <c r="AA20" s="41" t="s">
-        <v>31</v>
-      </c>
-      <c r="AB20" s="42" t="s">
+      <c r="AA20" s="40" t="s">
+        <v>32</v>
+      </c>
+      <c r="AB20" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="AC20" s="42" t="s">
+      <c r="AC20" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="AD20" s="48"/>
-      <c r="AE20" s="49"/>
-      <c r="AF20" s="49"/>
+      <c r="AD20" s="47"/>
+      <c r="AE20" s="48"/>
+      <c r="AF20" s="48"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="31">
+      <c r="A21" s="36">
         <v>10.0</v>
       </c>
-      <c r="B21" s="32">
+      <c r="B21" s="43">
         <v>0.5555555555555556</v>
       </c>
-      <c r="C21" s="33" t="s">
-        <v>32</v>
-      </c>
-      <c r="D21" s="33" t="s">
-        <v>21</v>
-      </c>
-      <c r="E21" s="33" t="s">
-        <v>15</v>
-      </c>
-      <c r="F21" s="33" t="s">
-        <v>19</v>
-      </c>
+      <c r="C21" s="44" t="s">
+        <v>33</v>
+      </c>
+      <c r="D21" s="44"/>
+      <c r="E21" s="44"/>
+      <c r="F21" s="44"/>
       <c r="G21" s="31">
         <v>10.0</v>
       </c>
@@ -2015,13 +2020,13 @@
         <v>0.5555555555555556</v>
       </c>
       <c r="I21" s="33" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J21" s="33" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K21" s="33" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L21" s="33" t="s">
         <v>19</v>
@@ -2032,16 +2037,16 @@
       <c r="N21" s="32">
         <v>0.5555555555555556</v>
       </c>
-      <c r="O21" s="50" t="s">
-        <v>35</v>
-      </c>
-      <c r="P21" s="51" t="s">
+      <c r="O21" s="49" t="s">
+        <v>36</v>
+      </c>
+      <c r="P21" s="50" t="s">
         <v>21</v>
       </c>
-      <c r="Q21" s="37" t="s">
-        <v>36</v>
-      </c>
-      <c r="R21" s="37" t="s">
+      <c r="Q21" s="38" t="s">
+        <v>37</v>
+      </c>
+      <c r="R21" s="38" t="s">
         <v>19</v>
       </c>
       <c r="S21" s="31">
@@ -2051,7 +2056,7 @@
         <v>0.5555555555555556</v>
       </c>
       <c r="U21" s="33" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V21" s="33" t="s">
         <v>21</v>
@@ -2067,13 +2072,13 @@
         <v>0.5555555555555556</v>
       </c>
       <c r="AA21" s="33" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="AB21" s="33" t="s">
         <v>21</v>
       </c>
       <c r="AC21" s="33" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="AD21" s="31"/>
       <c r="AE21" s="27"/>
@@ -2087,13 +2092,13 @@
         <v>0.5694444444444444</v>
       </c>
       <c r="C22" s="33" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D22" s="33" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E22" s="33" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F22" s="33" t="s">
         <v>19</v>
@@ -2101,27 +2106,27 @@
       <c r="G22" s="36">
         <v>11.0</v>
       </c>
-      <c r="H22" s="44">
+      <c r="H22" s="43">
         <v>0.5694444444444444</v>
       </c>
       <c r="I22" s="36"/>
       <c r="J22" s="36"/>
       <c r="K22" s="36"/>
       <c r="L22" s="36"/>
-      <c r="M22" s="31">
+      <c r="M22" s="24">
         <v>11.0</v>
       </c>
-      <c r="N22" s="32">
+      <c r="N22" s="25">
         <v>0.5694444444444444</v>
       </c>
-      <c r="O22" s="46" t="s">
-        <v>40</v>
+      <c r="O22" s="45" t="s">
+        <v>41</v>
       </c>
       <c r="P22" s="33" t="s">
         <v>21</v>
       </c>
       <c r="Q22" s="33" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="R22" s="31"/>
       <c r="S22" s="31">
@@ -2131,13 +2136,13 @@
         <v>0.5694444444444444</v>
       </c>
       <c r="U22" s="33" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="V22" s="33" t="s">
         <v>21</v>
       </c>
       <c r="W22" s="33" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="X22" s="33" t="s">
         <v>19</v>
@@ -2149,7 +2154,7 @@
         <v>0.5694444444444444</v>
       </c>
       <c r="AA22" s="33" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="AB22" s="33" t="s">
         <v>21</v>
@@ -2160,36 +2165,36 @@
       <c r="AD22" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="AE22" s="52"/>
-      <c r="AF22" s="52"/>
+      <c r="AE22" s="51"/>
+      <c r="AF22" s="51"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="37">
+      <c r="A23" s="38">
         <v>13.0</v>
       </c>
       <c r="B23" s="32">
         <v>0.5833333333333334</v>
       </c>
-      <c r="C23" s="37" t="s">
-        <v>43</v>
-      </c>
-      <c r="D23" s="37" t="s">
+      <c r="C23" s="38" t="s">
+        <v>44</v>
+      </c>
+      <c r="D23" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="E23" s="37" t="s">
-        <v>23</v>
-      </c>
-      <c r="F23" s="37" t="s">
+      <c r="E23" s="38" t="s">
+        <v>24</v>
+      </c>
+      <c r="F23" s="38" t="s">
         <v>19</v>
       </c>
       <c r="G23" s="36">
         <v>12.0</v>
       </c>
-      <c r="H23" s="44">
+      <c r="H23" s="43">
         <v>0.5833333333333334</v>
       </c>
       <c r="I23" s="36"/>
-      <c r="J23" s="53"/>
+      <c r="J23" s="52"/>
       <c r="K23" s="36"/>
       <c r="L23" s="36"/>
       <c r="M23" s="31">
@@ -2198,16 +2203,16 @@
       <c r="N23" s="32">
         <v>0.5833333333333334</v>
       </c>
-      <c r="O23" s="54" t="s">
-        <v>44</v>
-      </c>
-      <c r="P23" s="37" t="s">
+      <c r="O23" s="53" t="s">
+        <v>45</v>
+      </c>
+      <c r="P23" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="Q23" s="37" t="s">
+      <c r="Q23" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="R23" s="37" t="s">
+      <c r="R23" s="38" t="s">
         <v>19</v>
       </c>
       <c r="S23" s="31">
@@ -2217,7 +2222,7 @@
         <v>0.5833333333333334</v>
       </c>
       <c r="U23" s="33" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="V23" s="33" t="s">
         <v>21</v>
@@ -2234,16 +2239,16 @@
       <c r="Z23" s="32">
         <v>0.5833333333333334</v>
       </c>
-      <c r="AA23" s="37" t="s">
-        <v>46</v>
-      </c>
-      <c r="AB23" s="37" t="s">
+      <c r="AA23" s="38" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB23" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="AC23" s="37" t="s">
-        <v>23</v>
-      </c>
-      <c r="AD23" s="50"/>
+      <c r="AC23" s="38" t="s">
+        <v>24</v>
+      </c>
+      <c r="AD23" s="49"/>
       <c r="AE23" s="27"/>
       <c r="AF23" s="27"/>
     </row>
@@ -2255,13 +2260,13 @@
         <v>0.5972222222222222</v>
       </c>
       <c r="C24" s="33" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D24" s="33" t="s">
         <v>21</v>
       </c>
       <c r="E24" s="33" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F24" s="33" t="s">
         <v>19</v>
@@ -2273,13 +2278,13 @@
         <v>0.5972222222222222</v>
       </c>
       <c r="I24" s="33" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J24" s="33" t="s">
         <v>21</v>
       </c>
       <c r="K24" s="33" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L24" s="33" t="s">
         <v>19</v>
@@ -2290,16 +2295,16 @@
       <c r="N24" s="32">
         <v>0.5972222222222222</v>
       </c>
-      <c r="O24" s="37" t="s">
-        <v>49</v>
-      </c>
-      <c r="P24" s="37" t="s">
+      <c r="O24" s="38" t="s">
+        <v>50</v>
+      </c>
+      <c r="P24" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="Q24" s="37" t="s">
+      <c r="Q24" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="R24" s="37" t="s">
+      <c r="R24" s="38" t="s">
         <v>19</v>
       </c>
       <c r="S24" s="31">
@@ -2309,13 +2314,13 @@
         <v>0.5972222222222222</v>
       </c>
       <c r="U24" s="33" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="V24" s="33" t="s">
         <v>21</v>
       </c>
       <c r="W24" s="33" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="X24" s="33" t="s">
         <v>19</v>
@@ -2323,7 +2328,7 @@
       <c r="Y24" s="36">
         <v>13.0</v>
       </c>
-      <c r="Z24" s="44">
+      <c r="Z24" s="43">
         <v>0.5972222222222222</v>
       </c>
       <c r="AA24" s="36"/>
@@ -2337,7 +2342,7 @@
       <c r="A25" s="36">
         <v>14.0</v>
       </c>
-      <c r="B25" s="44">
+      <c r="B25" s="43">
         <v>0.6111111111111112</v>
       </c>
       <c r="C25" s="36"/>
@@ -2351,13 +2356,13 @@
         <v>0.6111111111111112</v>
       </c>
       <c r="I25" s="33" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="J25" s="33" t="s">
         <v>21</v>
       </c>
       <c r="K25" s="33" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L25" s="33" t="s">
         <v>19</v>
@@ -2369,7 +2374,7 @@
         <v>0.6111111111111112</v>
       </c>
       <c r="O25" s="33" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="P25" s="33" t="s">
         <v>21</v>
@@ -2385,7 +2390,7 @@
         <v>0.6111111111111112</v>
       </c>
       <c r="U25" s="33" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="V25" s="33" t="s">
         <v>21</v>
@@ -2403,13 +2408,13 @@
         <v>0.6111111111111112</v>
       </c>
       <c r="AA25" s="33" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="AB25" s="33" t="s">
         <v>21</v>
       </c>
       <c r="AC25" s="33" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="AD25" s="33" t="s">
         <v>19</v>
@@ -2421,12 +2426,12 @@
       <c r="A26" s="36">
         <v>15.0</v>
       </c>
-      <c r="B26" s="44">
+      <c r="B26" s="43">
         <v>0.625</v>
       </c>
-      <c r="C26" s="45"/>
-      <c r="D26" s="45"/>
-      <c r="E26" s="45"/>
+      <c r="C26" s="44"/>
+      <c r="D26" s="44"/>
+      <c r="E26" s="44"/>
       <c r="F26" s="36"/>
       <c r="G26" s="31">
         <v>15.0</v>
@@ -2435,13 +2440,13 @@
         <v>0.625</v>
       </c>
       <c r="I26" s="33" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J26" s="33" t="s">
         <v>21</v>
       </c>
       <c r="K26" s="33" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L26" s="33" t="s">
         <v>19</v>
@@ -2453,7 +2458,7 @@
         <v>0.625</v>
       </c>
       <c r="O26" s="33" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="P26" s="33" t="s">
         <v>21</v>
@@ -2469,13 +2474,13 @@
         <v>0.625</v>
       </c>
       <c r="U26" s="33" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="V26" s="33" t="s">
         <v>21</v>
       </c>
       <c r="W26" s="33" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="X26" s="33" t="s">
         <v>19</v>
@@ -2487,7 +2492,7 @@
         <v>0.625</v>
       </c>
       <c r="AA26" s="33" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="AB26" s="33" t="s">
         <v>21</v>
@@ -2496,22 +2501,26 @@
         <v>15</v>
       </c>
       <c r="AD26" s="33" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="AE26" s="27"/>
       <c r="AF26" s="27"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="22">
+      <c r="A27" s="31">
         <v>16.0</v>
       </c>
-      <c r="B27" s="23">
+      <c r="B27" s="32">
         <v>0.6388888888888888</v>
       </c>
-      <c r="C27" s="28"/>
-      <c r="D27" s="28"/>
-      <c r="E27" s="28"/>
-      <c r="F27" s="28"/>
+      <c r="C27" s="33" t="s">
+        <v>61</v>
+      </c>
+      <c r="D27" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="E27" s="33"/>
+      <c r="F27" s="33"/>
       <c r="G27" s="31">
         <v>16.0</v>
       </c>
@@ -2519,13 +2528,13 @@
         <v>0.6388888888888888</v>
       </c>
       <c r="I27" s="33" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J27" s="33" t="s">
         <v>21</v>
       </c>
       <c r="K27" s="33" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L27" s="33" t="s">
         <v>19</v>
@@ -2537,7 +2546,7 @@
         <v>0.6388888888888888</v>
       </c>
       <c r="O27" s="33" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="P27" s="33" t="s">
         <v>21</v>
@@ -2551,7 +2560,7 @@
       <c r="S27" s="36">
         <v>16.0</v>
       </c>
-      <c r="T27" s="44">
+      <c r="T27" s="43">
         <v>0.6388888888888888</v>
       </c>
       <c r="U27" s="36"/>
@@ -2565,13 +2574,13 @@
         <v>0.6388888888888888</v>
       </c>
       <c r="AA27" s="33" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="AB27" s="33" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="AC27" s="33" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="AD27" s="33" t="s">
         <v>19</v>
@@ -2587,13 +2596,13 @@
         <v>0.6527777777777778</v>
       </c>
       <c r="C28" s="33" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D28" s="33" t="s">
         <v>21</v>
       </c>
       <c r="E28" s="33" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F28" s="33" t="s">
         <v>19</v>
@@ -2605,13 +2614,13 @@
         <v>0.6527777777777778</v>
       </c>
       <c r="I28" s="33" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="J28" s="33" t="s">
         <v>21</v>
       </c>
       <c r="K28" s="33" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L28" s="33" t="s">
         <v>19</v>
@@ -2622,22 +2631,22 @@
       <c r="N28" s="32">
         <v>0.6527777777777778</v>
       </c>
-      <c r="O28" s="37" t="s">
-        <v>66</v>
-      </c>
-      <c r="P28" s="37" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q28" s="37" t="s">
+      <c r="O28" s="38" t="s">
+        <v>68</v>
+      </c>
+      <c r="P28" s="38" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q28" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="R28" s="55" t="s">
+      <c r="R28" s="54" t="s">
         <v>19</v>
       </c>
       <c r="S28" s="36">
         <v>17.0</v>
       </c>
-      <c r="T28" s="44">
+      <c r="T28" s="43">
         <v>0.6527777777777778</v>
       </c>
       <c r="U28" s="36"/>
@@ -2651,7 +2660,7 @@
         <v>0.6527777777777778</v>
       </c>
       <c r="AA28" s="33" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="AB28" s="33" t="s">
         <v>21</v>
@@ -2673,13 +2682,13 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="C29" s="33" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D29" s="33" t="s">
         <v>21</v>
       </c>
       <c r="E29" s="33" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F29" s="33" t="s">
         <v>19</v>
@@ -2687,7 +2696,7 @@
       <c r="G29" s="36">
         <v>18.0</v>
       </c>
-      <c r="H29" s="44">
+      <c r="H29" s="43">
         <v>0.6666666666666666</v>
       </c>
       <c r="I29" s="36"/>
@@ -2701,33 +2710,33 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="O29" s="33" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="P29" s="33" t="s">
         <v>21</v>
       </c>
       <c r="Q29" s="33" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="R29" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="S29" s="37">
+      <c r="S29" s="38">
         <v>18.0</v>
       </c>
-      <c r="T29" s="38">
+      <c r="T29" s="55">
         <v>0.6666666666666666</v>
       </c>
-      <c r="U29" s="47" t="s">
-        <v>72</v>
-      </c>
-      <c r="V29" s="47" t="s">
-        <v>67</v>
-      </c>
-      <c r="W29" s="47" t="s">
-        <v>23</v>
-      </c>
-      <c r="X29" s="55" t="s">
+      <c r="U29" s="46" t="s">
+        <v>74</v>
+      </c>
+      <c r="V29" s="46" t="s">
+        <v>69</v>
+      </c>
+      <c r="W29" s="46" t="s">
+        <v>24</v>
+      </c>
+      <c r="X29" s="54" t="s">
         <v>19</v>
       </c>
       <c r="Y29" s="31">
@@ -2736,14 +2745,14 @@
       <c r="Z29" s="32">
         <v>0.6666666666666666</v>
       </c>
-      <c r="AA29" s="47" t="s">
-        <v>73</v>
-      </c>
-      <c r="AB29" s="47" t="s">
+      <c r="AA29" s="46" t="s">
+        <v>75</v>
+      </c>
+      <c r="AB29" s="46" t="s">
         <v>21</v>
       </c>
-      <c r="AC29" s="47" t="s">
-        <v>23</v>
+      <c r="AC29" s="46" t="s">
+        <v>24</v>
       </c>
       <c r="AD29" s="56" t="s">
         <v>19</v>
@@ -2759,7 +2768,7 @@
         <v>0.6805555555555556</v>
       </c>
       <c r="C30" s="33" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D30" s="33" t="s">
         <v>21</v>
@@ -2775,13 +2784,13 @@
         <v>0.6805555555555556</v>
       </c>
       <c r="I30" s="33" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="J30" s="33" t="s">
         <v>21</v>
       </c>
       <c r="K30" s="33" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L30" s="33" t="s">
         <v>19</v>
@@ -2793,16 +2802,16 @@
         <v>0.6805555555555556</v>
       </c>
       <c r="O30" s="33" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="P30" s="33" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Q30" s="33" t="s">
         <v>15</v>
       </c>
       <c r="R30" s="33" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="S30" s="22">
         <v>19.0</v>
@@ -2835,7 +2844,7 @@
         <v>0.6944444444444444</v>
       </c>
       <c r="C31" s="33" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D31" s="33" t="s">
         <v>21</v>
@@ -2863,7 +2872,7 @@
         <v>0.6944444444444444</v>
       </c>
       <c r="O31" s="61" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="P31" s="62"/>
       <c r="Q31" s="62"/>
@@ -2919,7 +2928,7 @@
         <v>0.7083333333333334</v>
       </c>
       <c r="O32" s="61" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="P32" s="62"/>
       <c r="Q32" s="62"/>
@@ -2975,7 +2984,7 @@
         <v>0.7222222222222222</v>
       </c>
       <c r="O33" s="61" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="P33" s="62"/>
       <c r="Q33" s="62"/>
@@ -2997,7 +3006,7 @@
         <v>0.7222222222222222</v>
       </c>
       <c r="AA33" s="22" t="s">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="AB33" s="22"/>
       <c r="AC33" s="22"/>
@@ -3033,7 +3042,7 @@
         <v>0.7361111111111112</v>
       </c>
       <c r="O34" s="61" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="P34" s="62"/>
       <c r="Q34" s="62"/>
@@ -3089,7 +3098,7 @@
         <v>0.75</v>
       </c>
       <c r="O35" s="61" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="P35" s="62"/>
       <c r="Q35" s="62"/>
@@ -3145,7 +3154,7 @@
         <v>0.7638888888888888</v>
       </c>
       <c r="O36" s="61" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="P36" s="62"/>
       <c r="Q36" s="62"/>
@@ -3201,7 +3210,7 @@
         <v>0.7777777777777778</v>
       </c>
       <c r="O37" s="61" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="P37" s="62"/>
       <c r="Q37" s="62"/>
@@ -3257,7 +3266,7 @@
         <v>0.7916666666666666</v>
       </c>
       <c r="O38" s="61" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="P38" s="62"/>
       <c r="Q38" s="62"/>
@@ -3313,7 +3322,7 @@
         <v>0.8055555555555556</v>
       </c>
       <c r="O39" s="61" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="P39" s="62"/>
       <c r="Q39" s="62"/>
@@ -3369,7 +3378,7 @@
         <v>0.8194444444444444</v>
       </c>
       <c r="O40" s="61" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="P40" s="62"/>
       <c r="Q40" s="62"/>
@@ -3425,7 +3434,7 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="O41" s="61" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="P41" s="62"/>
       <c r="Q41" s="62"/>
@@ -3481,7 +3490,7 @@
         <v>0.8472222222222222</v>
       </c>
       <c r="O42" s="61" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="P42" s="62"/>
       <c r="Q42" s="62"/>
@@ -3537,7 +3546,7 @@
         <v>0.8611111111111112</v>
       </c>
       <c r="O43" s="69" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="P43" s="70"/>
       <c r="Q43" s="70"/>

</xml_diff>

<commit_message>
feat: enable multi-month schedule & waste booking audit for Jan-Oct 2026
</commit_message>
<xml_diff>
--- a/file_wisuda_4okt.xlsx
+++ b/file_wisuda_4okt.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="81">
   <si>
     <t xml:space="preserve">Graduation Schedule 
 </t>
@@ -406,14 +406,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FF00"/>
-        <bgColor rgb="FF00FF00"/>
+        <fgColor rgb="FFFF0000"/>
+        <bgColor rgb="FFFF0000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor rgb="FFFF0000"/>
+        <fgColor rgb="FF00FF00"/>
+        <bgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -563,7 +563,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="76">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -653,78 +653,87 @@
     <xf borderId="5" fillId="9" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="5" fillId="10" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="10" fontId="13" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf borderId="5" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf borderId="5" fillId="9" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="9" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="11" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="6" fillId="9" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf borderId="5" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
     <xf borderId="5" fillId="10" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="5" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="11" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="11" fontId="13" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf borderId="6" fillId="9" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="6" fillId="11" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="5" fillId="11" fontId="15" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="15" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="5" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="10" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="10" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="5" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf borderId="5" fillId="11" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="11" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="7" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="6" fillId="11" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="6" fillId="10" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="5" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="10" fontId="15" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="15" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="5" fillId="10" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="7" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="11" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="10" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="5" fillId="10" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="5" fillId="11" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="5" fillId="10" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="5" fillId="11" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="8" fillId="10" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="8" fillId="11" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -815,7 +824,7 @@
     <xdr:ext cx="209550" cy="142875"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image2.jpg"/>
+        <xdr:cNvPr id="0" name="image5.jpg"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -843,7 +852,7 @@
     <xdr:ext cx="209550" cy="142875"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image6.jpg"/>
+        <xdr:cNvPr id="0" name="image2.jpg"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -871,7 +880,7 @@
     <xdr:ext cx="209550" cy="142875"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image3.jpg"/>
+        <xdr:cNvPr id="0" name="image4.jpg"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -899,7 +908,7 @@
     <xdr:ext cx="209550" cy="142875"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image4.jpg"/>
+        <xdr:cNvPr id="0" name="image6.jpg"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -927,7 +936,7 @@
     <xdr:ext cx="209550" cy="142875"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="image5.jpg"/>
+        <xdr:cNvPr id="0" name="image3.jpg"/>
         <xdr:cNvPicPr preferRelativeResize="0"/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1771,22 +1780,22 @@
       <c r="AF17" s="27"/>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="31">
+      <c r="A18" s="24">
         <v>7.0</v>
       </c>
-      <c r="B18" s="32">
+      <c r="B18" s="25">
         <v>0.5</v>
       </c>
-      <c r="C18" s="33" t="s">
+      <c r="C18" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="D18" s="33" t="s">
+      <c r="D18" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="E18" s="33" t="s">
+      <c r="E18" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="F18" s="33" t="s">
+      <c r="F18" s="26" t="s">
         <v>19</v>
       </c>
       <c r="G18" s="22">
@@ -1839,44 +1848,44 @@
       <c r="B19" s="25">
         <v>0.5208333333333334</v>
       </c>
-      <c r="C19" s="33" t="s">
+      <c r="C19" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="D19" s="33" t="s">
+      <c r="D19" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="E19" s="33" t="s">
+      <c r="E19" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="F19" s="33" t="s">
+      <c r="F19" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="G19" s="34">
+      <c r="G19" s="31">
         <v>8.0</v>
       </c>
-      <c r="H19" s="35">
+      <c r="H19" s="32">
         <v>0.5208333333333334</v>
       </c>
-      <c r="I19" s="34"/>
-      <c r="J19" s="36"/>
-      <c r="K19" s="36"/>
-      <c r="L19" s="36"/>
+      <c r="I19" s="31"/>
+      <c r="J19" s="33"/>
+      <c r="K19" s="33"/>
+      <c r="L19" s="33"/>
       <c r="M19" s="29">
         <v>8.0</v>
       </c>
       <c r="N19" s="30">
         <v>0.5208333333333334</v>
       </c>
-      <c r="O19" s="37" t="s">
+      <c r="O19" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="P19" s="38" t="s">
+      <c r="P19" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="Q19" s="38" t="s">
+      <c r="Q19" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="R19" s="37" t="s">
+      <c r="R19" s="34" t="s">
         <v>19</v>
       </c>
       <c r="S19" s="24">
@@ -1885,16 +1894,16 @@
       <c r="T19" s="25">
         <v>0.5208333333333334</v>
       </c>
-      <c r="U19" s="39" t="s">
+      <c r="U19" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="V19" s="39" t="s">
+      <c r="V19" s="36" t="s">
         <v>21</v>
       </c>
-      <c r="W19" s="39" t="s">
+      <c r="W19" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="X19" s="39" t="s">
+      <c r="X19" s="36" t="s">
         <v>19</v>
       </c>
       <c r="Y19" s="29">
@@ -1903,82 +1912,82 @@
       <c r="Z19" s="30">
         <v>0.5208333333333334</v>
       </c>
-      <c r="AA19" s="40" t="s">
+      <c r="AA19" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="AB19" s="41" t="s">
+      <c r="AB19" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="AC19" s="41" t="s">
+      <c r="AC19" s="38" t="s">
         <v>15</v>
       </c>
-      <c r="AD19" s="38" t="s">
+      <c r="AD19" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="AE19" s="42"/>
-      <c r="AF19" s="42"/>
+      <c r="AE19" s="40"/>
+      <c r="AF19" s="40"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="31">
+      <c r="A20" s="24">
         <v>9.0</v>
       </c>
-      <c r="B20" s="32">
+      <c r="B20" s="25">
         <v>0.5416666666666666</v>
       </c>
-      <c r="C20" s="33" t="s">
+      <c r="C20" s="41" t="s">
         <v>29</v>
       </c>
-      <c r="D20" s="33" t="s">
+      <c r="D20" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="E20" s="33" t="s">
+      <c r="E20" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="F20" s="33"/>
-      <c r="G20" s="36">
+      <c r="F20" s="41"/>
+      <c r="G20" s="33">
         <v>9.0</v>
       </c>
-      <c r="H20" s="43">
+      <c r="H20" s="42">
         <v>0.5416666666666666</v>
       </c>
-      <c r="I20" s="44"/>
-      <c r="J20" s="44"/>
-      <c r="K20" s="44"/>
-      <c r="L20" s="44"/>
-      <c r="M20" s="31">
+      <c r="I20" s="43"/>
+      <c r="J20" s="43"/>
+      <c r="K20" s="43"/>
+      <c r="L20" s="43"/>
+      <c r="M20" s="24">
         <v>9.0</v>
       </c>
-      <c r="N20" s="32">
+      <c r="N20" s="25">
         <v>0.5416666666666666</v>
       </c>
-      <c r="O20" s="45" t="s">
+      <c r="O20" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="P20" s="46" t="s">
+      <c r="P20" s="45" t="s">
         <v>21</v>
       </c>
-      <c r="Q20" s="46" t="s">
+      <c r="Q20" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="R20" s="33" t="s">
+      <c r="R20" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="S20" s="31">
+      <c r="S20" s="24">
         <v>9.0</v>
       </c>
-      <c r="T20" s="32">
+      <c r="T20" s="25">
         <v>0.5416666666666666</v>
       </c>
-      <c r="U20" s="33" t="s">
+      <c r="U20" s="41" t="s">
         <v>31</v>
       </c>
-      <c r="V20" s="33" t="s">
+      <c r="V20" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="W20" s="33" t="s">
+      <c r="W20" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="X20" s="33" t="s">
+      <c r="X20" s="41" t="s">
         <v>19</v>
       </c>
       <c r="Y20" s="29">
@@ -1987,13 +1996,13 @@
       <c r="Z20" s="30">
         <v>0.5416666666666666</v>
       </c>
-      <c r="AA20" s="40" t="s">
+      <c r="AA20" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="AB20" s="41" t="s">
+      <c r="AB20" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="AC20" s="41" t="s">
+      <c r="AC20" s="38" t="s">
         <v>15</v>
       </c>
       <c r="AD20" s="47"/>
@@ -2001,816 +2010,814 @@
       <c r="AF20" s="48"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="36">
+      <c r="A21" s="33">
         <v>10.0</v>
       </c>
-      <c r="B21" s="43">
+      <c r="B21" s="42">
         <v>0.5555555555555556</v>
       </c>
-      <c r="C21" s="44" t="s">
+      <c r="C21" s="43" t="s">
         <v>33</v>
       </c>
-      <c r="D21" s="44"/>
-      <c r="E21" s="44"/>
-      <c r="F21" s="44"/>
-      <c r="G21" s="31">
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="49">
         <v>10.0</v>
       </c>
-      <c r="H21" s="32">
+      <c r="H21" s="50">
         <v>0.5555555555555556</v>
       </c>
-      <c r="I21" s="33" t="s">
+      <c r="I21" s="41" t="s">
         <v>34</v>
       </c>
-      <c r="J21" s="33" t="s">
+      <c r="J21" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="K21" s="33" t="s">
+      <c r="K21" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="L21" s="33" t="s">
+      <c r="L21" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="M21" s="31">
+      <c r="M21" s="49">
         <v>10.0</v>
       </c>
-      <c r="N21" s="32">
+      <c r="N21" s="50">
         <v>0.5555555555555556</v>
       </c>
-      <c r="O21" s="49" t="s">
+      <c r="O21" s="51" t="s">
         <v>36</v>
       </c>
-      <c r="P21" s="50" t="s">
+      <c r="P21" s="52" t="s">
         <v>21</v>
       </c>
-      <c r="Q21" s="38" t="s">
+      <c r="Q21" s="39" t="s">
         <v>37</v>
       </c>
-      <c r="R21" s="38" t="s">
+      <c r="R21" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="S21" s="31">
+      <c r="S21" s="49">
         <v>10.0</v>
       </c>
-      <c r="T21" s="32">
+      <c r="T21" s="50">
         <v>0.5555555555555556</v>
       </c>
-      <c r="U21" s="33" t="s">
+      <c r="U21" s="41" t="s">
         <v>38</v>
       </c>
-      <c r="V21" s="33" t="s">
+      <c r="V21" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="W21" s="33" t="s">
+      <c r="W21" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="X21" s="31"/>
-      <c r="Y21" s="31">
+      <c r="X21" s="49"/>
+      <c r="Y21" s="24">
         <v>10.0</v>
       </c>
-      <c r="Z21" s="32">
+      <c r="Z21" s="25">
         <v>0.5555555555555556</v>
       </c>
-      <c r="AA21" s="33" t="s">
+      <c r="AA21" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="AB21" s="33" t="s">
+      <c r="AB21" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="AC21" s="33" t="s">
+      <c r="AC21" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="AD21" s="31"/>
+      <c r="AD21" s="49"/>
       <c r="AE21" s="27"/>
       <c r="AF21" s="27"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="31">
+      <c r="A22" s="49">
         <v>11.0</v>
       </c>
-      <c r="B22" s="32">
+      <c r="B22" s="50">
         <v>0.5694444444444444</v>
       </c>
-      <c r="C22" s="33" t="s">
+      <c r="C22" s="41" t="s">
         <v>34</v>
       </c>
-      <c r="D22" s="33" t="s">
+      <c r="D22" s="41" t="s">
         <v>40</v>
       </c>
-      <c r="E22" s="33" t="s">
+      <c r="E22" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="F22" s="33" t="s">
+      <c r="F22" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="G22" s="36">
+      <c r="G22" s="33">
         <v>11.0</v>
       </c>
-      <c r="H22" s="43">
+      <c r="H22" s="42">
         <v>0.5694444444444444</v>
       </c>
-      <c r="I22" s="36"/>
-      <c r="J22" s="36"/>
-      <c r="K22" s="36"/>
-      <c r="L22" s="36"/>
+      <c r="I22" s="33"/>
+      <c r="J22" s="33"/>
+      <c r="K22" s="33"/>
+      <c r="L22" s="33"/>
       <c r="M22" s="24">
         <v>11.0</v>
       </c>
       <c r="N22" s="25">
         <v>0.5694444444444444</v>
       </c>
-      <c r="O22" s="45" t="s">
+      <c r="O22" s="53" t="s">
         <v>41</v>
       </c>
-      <c r="P22" s="33" t="s">
+      <c r="P22" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="Q22" s="33" t="s">
+      <c r="Q22" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="R22" s="31"/>
-      <c r="S22" s="31">
+      <c r="R22" s="49"/>
+      <c r="S22" s="49">
         <v>11.0</v>
       </c>
-      <c r="T22" s="32">
+      <c r="T22" s="50">
         <v>0.5694444444444444</v>
       </c>
-      <c r="U22" s="33" t="s">
+      <c r="U22" s="41" t="s">
         <v>42</v>
       </c>
-      <c r="V22" s="33" t="s">
+      <c r="V22" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="W22" s="33" t="s">
+      <c r="W22" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="X22" s="33" t="s">
+      <c r="X22" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="Y22" s="31">
+      <c r="Y22" s="49">
         <v>11.0</v>
       </c>
-      <c r="Z22" s="32">
+      <c r="Z22" s="50">
         <v>0.5694444444444444</v>
       </c>
-      <c r="AA22" s="33" t="s">
+      <c r="AA22" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="AB22" s="33" t="s">
+      <c r="AB22" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="AC22" s="33" t="s">
+      <c r="AC22" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="AD22" s="33" t="s">
+      <c r="AD22" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="AE22" s="51"/>
-      <c r="AF22" s="51"/>
+      <c r="AE22" s="54"/>
+      <c r="AF22" s="54"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="38">
+      <c r="A23" s="39">
         <v>13.0</v>
       </c>
-      <c r="B23" s="32">
+      <c r="B23" s="50">
         <v>0.5833333333333334</v>
       </c>
-      <c r="C23" s="38" t="s">
+      <c r="C23" s="39" t="s">
         <v>44</v>
       </c>
-      <c r="D23" s="38" t="s">
+      <c r="D23" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="E23" s="38" t="s">
+      <c r="E23" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="F23" s="38" t="s">
+      <c r="F23" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="G23" s="36">
+      <c r="G23" s="33">
         <v>12.0</v>
       </c>
-      <c r="H23" s="43">
+      <c r="H23" s="42">
         <v>0.5833333333333334</v>
       </c>
-      <c r="I23" s="36"/>
-      <c r="J23" s="52"/>
-      <c r="K23" s="36"/>
-      <c r="L23" s="36"/>
-      <c r="M23" s="31">
+      <c r="I23" s="33"/>
+      <c r="J23" s="55"/>
+      <c r="K23" s="33"/>
+      <c r="L23" s="33"/>
+      <c r="M23" s="49">
         <v>12.0</v>
       </c>
-      <c r="N23" s="32">
+      <c r="N23" s="50">
         <v>0.5833333333333334</v>
       </c>
-      <c r="O23" s="53" t="s">
+      <c r="O23" s="56" t="s">
         <v>45</v>
       </c>
-      <c r="P23" s="38" t="s">
+      <c r="P23" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="Q23" s="38" t="s">
+      <c r="Q23" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="R23" s="38" t="s">
+      <c r="R23" s="39"/>
+      <c r="S23" s="49">
+        <v>12.0</v>
+      </c>
+      <c r="T23" s="50">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="U23" s="41" t="s">
+        <v>46</v>
+      </c>
+      <c r="V23" s="41" t="s">
+        <v>21</v>
+      </c>
+      <c r="W23" s="41" t="s">
+        <v>15</v>
+      </c>
+      <c r="X23" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="S23" s="31">
+      <c r="Y23" s="49">
         <v>12.0</v>
       </c>
-      <c r="T23" s="32">
+      <c r="Z23" s="50">
         <v>0.5833333333333334</v>
       </c>
-      <c r="U23" s="33" t="s">
-        <v>46</v>
-      </c>
-      <c r="V23" s="33" t="s">
+      <c r="AA23" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB23" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="W23" s="33" t="s">
-        <v>15</v>
-      </c>
-      <c r="X23" s="33" t="s">
-        <v>19</v>
-      </c>
-      <c r="Y23" s="31">
-        <v>12.0</v>
-      </c>
-      <c r="Z23" s="32">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="AA23" s="38" t="s">
-        <v>47</v>
-      </c>
-      <c r="AB23" s="38" t="s">
-        <v>21</v>
-      </c>
-      <c r="AC23" s="38" t="s">
+      <c r="AC23" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="AD23" s="49"/>
+      <c r="AD23" s="51"/>
       <c r="AE23" s="27"/>
       <c r="AF23" s="27"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="33">
+      <c r="A24" s="41">
         <v>14.0</v>
       </c>
-      <c r="B24" s="32">
+      <c r="B24" s="50">
         <v>0.5972222222222222</v>
       </c>
-      <c r="C24" s="33" t="s">
+      <c r="C24" s="41" t="s">
         <v>48</v>
       </c>
-      <c r="D24" s="33" t="s">
+      <c r="D24" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="E24" s="33" t="s">
+      <c r="E24" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="F24" s="33" t="s">
+      <c r="F24" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="G24" s="31">
+      <c r="G24" s="49">
         <v>13.0</v>
       </c>
-      <c r="H24" s="32">
+      <c r="H24" s="50">
         <v>0.5972222222222222</v>
       </c>
-      <c r="I24" s="33" t="s">
+      <c r="I24" s="41" t="s">
         <v>49</v>
       </c>
-      <c r="J24" s="33" t="s">
+      <c r="J24" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="K24" s="33" t="s">
+      <c r="K24" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="L24" s="33" t="s">
+      <c r="L24" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="M24" s="31">
+      <c r="M24" s="49">
         <v>13.0</v>
       </c>
-      <c r="N24" s="32">
+      <c r="N24" s="50">
         <v>0.5972222222222222</v>
       </c>
-      <c r="O24" s="38" t="s">
+      <c r="O24" s="39" t="s">
         <v>50</v>
       </c>
-      <c r="P24" s="38" t="s">
+      <c r="P24" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="Q24" s="38" t="s">
+      <c r="Q24" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="R24" s="38" t="s">
+      <c r="R24" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="S24" s="31">
+      <c r="S24" s="49">
         <v>13.0</v>
       </c>
-      <c r="T24" s="32">
+      <c r="T24" s="50">
         <v>0.5972222222222222</v>
       </c>
-      <c r="U24" s="33" t="s">
+      <c r="U24" s="41" t="s">
         <v>51</v>
       </c>
-      <c r="V24" s="33" t="s">
+      <c r="V24" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="W24" s="33" t="s">
+      <c r="W24" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="X24" s="33" t="s">
+      <c r="X24" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="Y24" s="36">
+      <c r="Y24" s="33">
         <v>13.0</v>
       </c>
-      <c r="Z24" s="43">
+      <c r="Z24" s="42">
         <v>0.5972222222222222</v>
       </c>
-      <c r="AA24" s="36"/>
-      <c r="AB24" s="36"/>
-      <c r="AC24" s="36"/>
-      <c r="AD24" s="36"/>
+      <c r="AA24" s="33"/>
+      <c r="AB24" s="33"/>
+      <c r="AC24" s="33"/>
+      <c r="AD24" s="33"/>
       <c r="AE24" s="27"/>
       <c r="AF24" s="27"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="36">
+      <c r="A25" s="33">
         <v>14.0</v>
       </c>
-      <c r="B25" s="43">
+      <c r="B25" s="42">
         <v>0.6111111111111112</v>
       </c>
-      <c r="C25" s="36"/>
-      <c r="D25" s="36"/>
-      <c r="E25" s="36"/>
-      <c r="F25" s="36"/>
-      <c r="G25" s="31">
+      <c r="C25" s="33"/>
+      <c r="D25" s="33"/>
+      <c r="E25" s="33"/>
+      <c r="F25" s="33"/>
+      <c r="G25" s="49">
         <v>14.0</v>
       </c>
-      <c r="H25" s="32">
+      <c r="H25" s="50">
         <v>0.6111111111111112</v>
       </c>
-      <c r="I25" s="33" t="s">
+      <c r="I25" s="41" t="s">
         <v>52</v>
       </c>
-      <c r="J25" s="33" t="s">
+      <c r="J25" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="K25" s="33" t="s">
+      <c r="K25" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="L25" s="33" t="s">
+      <c r="L25" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="M25" s="31">
+      <c r="M25" s="49">
         <v>14.0</v>
       </c>
-      <c r="N25" s="32">
+      <c r="N25" s="50">
         <v>0.6111111111111112</v>
       </c>
-      <c r="O25" s="33" t="s">
+      <c r="O25" s="41" t="s">
         <v>53</v>
       </c>
-      <c r="P25" s="33" t="s">
+      <c r="P25" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="Q25" s="33" t="s">
+      <c r="Q25" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="R25" s="31"/>
-      <c r="S25" s="31">
+      <c r="R25" s="49"/>
+      <c r="S25" s="49">
         <v>14.0</v>
       </c>
-      <c r="T25" s="32">
+      <c r="T25" s="50">
         <v>0.6111111111111112</v>
       </c>
-      <c r="U25" s="33" t="s">
+      <c r="U25" s="41" t="s">
         <v>54</v>
       </c>
-      <c r="V25" s="33" t="s">
+      <c r="V25" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="W25" s="33" t="s">
+      <c r="W25" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="X25" s="33" t="s">
+      <c r="X25" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="Y25" s="31">
+      <c r="Y25" s="49">
         <v>14.0</v>
       </c>
-      <c r="Z25" s="32">
+      <c r="Z25" s="50">
         <v>0.6111111111111112</v>
       </c>
-      <c r="AA25" s="33" t="s">
+      <c r="AA25" s="41" t="s">
         <v>55</v>
       </c>
-      <c r="AB25" s="33" t="s">
+      <c r="AB25" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="AC25" s="33" t="s">
+      <c r="AC25" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="AD25" s="33" t="s">
+      <c r="AD25" s="41" t="s">
         <v>19</v>
       </c>
       <c r="AE25" s="27"/>
       <c r="AF25" s="27"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="36">
+      <c r="A26" s="33">
         <v>15.0</v>
       </c>
-      <c r="B26" s="43">
+      <c r="B26" s="42">
         <v>0.625</v>
       </c>
-      <c r="C26" s="44"/>
-      <c r="D26" s="44"/>
-      <c r="E26" s="44"/>
-      <c r="F26" s="36"/>
-      <c r="G26" s="31">
+      <c r="C26" s="43"/>
+      <c r="D26" s="43"/>
+      <c r="E26" s="43"/>
+      <c r="F26" s="33"/>
+      <c r="G26" s="49">
         <v>15.0</v>
       </c>
-      <c r="H26" s="32">
+      <c r="H26" s="50">
         <v>0.625</v>
       </c>
-      <c r="I26" s="33" t="s">
+      <c r="I26" s="41" t="s">
         <v>56</v>
       </c>
-      <c r="J26" s="33" t="s">
+      <c r="J26" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="K26" s="33" t="s">
+      <c r="K26" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="L26" s="33" t="s">
+      <c r="L26" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="M26" s="31">
+      <c r="M26" s="49">
         <v>15.0</v>
       </c>
-      <c r="N26" s="32">
+      <c r="N26" s="50">
         <v>0.625</v>
       </c>
-      <c r="O26" s="33" t="s">
+      <c r="O26" s="41" t="s">
         <v>57</v>
       </c>
-      <c r="P26" s="33" t="s">
+      <c r="P26" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="Q26" s="33" t="s">
+      <c r="Q26" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="R26" s="31"/>
-      <c r="S26" s="31">
+      <c r="R26" s="49"/>
+      <c r="S26" s="49">
         <v>15.0</v>
       </c>
-      <c r="T26" s="32">
+      <c r="T26" s="50">
         <v>0.625</v>
       </c>
-      <c r="U26" s="33" t="s">
+      <c r="U26" s="41" t="s">
         <v>58</v>
       </c>
-      <c r="V26" s="33" t="s">
+      <c r="V26" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="W26" s="33" t="s">
+      <c r="W26" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="X26" s="33" t="s">
+      <c r="X26" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="Y26" s="31">
+      <c r="Y26" s="49">
         <v>15.0</v>
       </c>
-      <c r="Z26" s="32">
+      <c r="Z26" s="50">
         <v>0.625</v>
       </c>
-      <c r="AA26" s="33" t="s">
+      <c r="AA26" s="41" t="s">
         <v>59</v>
       </c>
-      <c r="AB26" s="33" t="s">
+      <c r="AB26" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="AC26" s="33" t="s">
+      <c r="AC26" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="AD26" s="33" t="s">
+      <c r="AD26" s="41" t="s">
         <v>60</v>
       </c>
       <c r="AE26" s="27"/>
       <c r="AF26" s="27"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="31">
+      <c r="A27" s="49">
         <v>16.0</v>
       </c>
-      <c r="B27" s="32">
+      <c r="B27" s="50">
         <v>0.6388888888888888</v>
       </c>
-      <c r="C27" s="33" t="s">
+      <c r="C27" s="41" t="s">
         <v>61</v>
       </c>
-      <c r="D27" s="33" t="s">
+      <c r="D27" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="E27" s="33"/>
-      <c r="F27" s="33"/>
-      <c r="G27" s="31">
+      <c r="E27" s="41"/>
+      <c r="F27" s="41"/>
+      <c r="G27" s="49">
         <v>16.0</v>
       </c>
-      <c r="H27" s="32">
+      <c r="H27" s="50">
         <v>0.6388888888888888</v>
       </c>
-      <c r="I27" s="33" t="s">
+      <c r="I27" s="41" t="s">
         <v>62</v>
       </c>
-      <c r="J27" s="33" t="s">
+      <c r="J27" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="K27" s="33" t="s">
+      <c r="K27" s="41" t="s">
         <v>63</v>
       </c>
-      <c r="L27" s="33" t="s">
+      <c r="L27" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="M27" s="31">
+      <c r="M27" s="49">
         <v>16.0</v>
       </c>
-      <c r="N27" s="32">
+      <c r="N27" s="50">
         <v>0.6388888888888888</v>
       </c>
-      <c r="O27" s="33" t="s">
+      <c r="O27" s="41" t="s">
         <v>64</v>
       </c>
-      <c r="P27" s="33" t="s">
+      <c r="P27" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="Q27" s="33" t="s">
+      <c r="Q27" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="R27" s="33" t="s">
+      <c r="R27" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="S27" s="36">
+      <c r="S27" s="33">
         <v>16.0</v>
       </c>
-      <c r="T27" s="43">
+      <c r="T27" s="42">
         <v>0.6388888888888888</v>
       </c>
-      <c r="U27" s="36"/>
-      <c r="V27" s="36"/>
-      <c r="W27" s="36"/>
-      <c r="X27" s="36"/>
-      <c r="Y27" s="31">
+      <c r="U27" s="33"/>
+      <c r="V27" s="33"/>
+      <c r="W27" s="33"/>
+      <c r="X27" s="33"/>
+      <c r="Y27" s="49">
         <v>16.0</v>
       </c>
-      <c r="Z27" s="32">
+      <c r="Z27" s="50">
         <v>0.6388888888888888</v>
       </c>
-      <c r="AA27" s="33" t="s">
+      <c r="AA27" s="41" t="s">
         <v>65</v>
       </c>
-      <c r="AB27" s="33" t="s">
+      <c r="AB27" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="AC27" s="33" t="s">
+      <c r="AC27" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="AD27" s="33" t="s">
+      <c r="AD27" s="41" t="s">
         <v>19</v>
       </c>
       <c r="AE27" s="27"/>
       <c r="AF27" s="27"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="31">
+      <c r="A28" s="49">
         <v>17.0</v>
       </c>
-      <c r="B28" s="32">
+      <c r="B28" s="50">
         <v>0.6527777777777778</v>
       </c>
-      <c r="C28" s="33" t="s">
+      <c r="C28" s="41" t="s">
         <v>66</v>
       </c>
-      <c r="D28" s="33" t="s">
+      <c r="D28" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="E28" s="33" t="s">
+      <c r="E28" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="F28" s="33" t="s">
+      <c r="F28" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="G28" s="31">
+      <c r="G28" s="49">
         <v>17.0</v>
       </c>
-      <c r="H28" s="32">
+      <c r="H28" s="50">
         <v>0.6527777777777778</v>
       </c>
-      <c r="I28" s="33" t="s">
+      <c r="I28" s="41" t="s">
         <v>67</v>
       </c>
-      <c r="J28" s="33" t="s">
+      <c r="J28" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="K28" s="33" t="s">
+      <c r="K28" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="L28" s="33" t="s">
+      <c r="L28" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="M28" s="31">
+      <c r="M28" s="49">
         <v>17.0</v>
       </c>
-      <c r="N28" s="32">
+      <c r="N28" s="50">
         <v>0.6527777777777778</v>
       </c>
-      <c r="O28" s="38" t="s">
+      <c r="O28" s="39" t="s">
         <v>68</v>
       </c>
-      <c r="P28" s="38" t="s">
+      <c r="P28" s="39" t="s">
         <v>69</v>
       </c>
-      <c r="Q28" s="38" t="s">
+      <c r="Q28" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="R28" s="54" t="s">
+      <c r="R28" s="57" t="s">
         <v>19</v>
       </c>
-      <c r="S28" s="36">
+      <c r="S28" s="33">
         <v>17.0</v>
       </c>
-      <c r="T28" s="43">
+      <c r="T28" s="42">
         <v>0.6527777777777778</v>
       </c>
-      <c r="U28" s="36"/>
-      <c r="V28" s="36"/>
-      <c r="W28" s="36"/>
-      <c r="X28" s="36"/>
-      <c r="Y28" s="31">
+      <c r="U28" s="33"/>
+      <c r="V28" s="33"/>
+      <c r="W28" s="33"/>
+      <c r="X28" s="33"/>
+      <c r="Y28" s="49">
         <v>17.0</v>
       </c>
-      <c r="Z28" s="32">
+      <c r="Z28" s="50">
         <v>0.6527777777777778</v>
       </c>
-      <c r="AA28" s="33" t="s">
+      <c r="AA28" s="41" t="s">
         <v>70</v>
       </c>
-      <c r="AB28" s="33" t="s">
+      <c r="AB28" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="AC28" s="33" t="s">
+      <c r="AC28" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="AD28" s="33" t="s">
+      <c r="AD28" s="41" t="s">
         <v>19</v>
       </c>
       <c r="AE28" s="27"/>
       <c r="AF28" s="27"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="31">
+      <c r="A29" s="49">
         <v>18.0</v>
       </c>
-      <c r="B29" s="32">
+      <c r="B29" s="50">
         <v>0.6666666666666666</v>
       </c>
-      <c r="C29" s="33" t="s">
+      <c r="C29" s="41" t="s">
         <v>71</v>
       </c>
-      <c r="D29" s="33" t="s">
+      <c r="D29" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="E29" s="33" t="s">
+      <c r="E29" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="F29" s="33" t="s">
+      <c r="F29" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="G29" s="36">
+      <c r="G29" s="33">
         <v>18.0</v>
       </c>
-      <c r="H29" s="43">
+      <c r="H29" s="42">
         <v>0.6666666666666666</v>
       </c>
-      <c r="I29" s="36"/>
-      <c r="J29" s="36"/>
-      <c r="K29" s="36"/>
-      <c r="L29" s="36"/>
-      <c r="M29" s="31">
+      <c r="I29" s="33"/>
+      <c r="J29" s="33"/>
+      <c r="K29" s="33"/>
+      <c r="L29" s="33"/>
+      <c r="M29" s="49">
         <v>18.0</v>
       </c>
-      <c r="N29" s="32">
+      <c r="N29" s="50">
         <v>0.6666666666666666</v>
       </c>
-      <c r="O29" s="33" t="s">
+      <c r="O29" s="41" t="s">
         <v>72</v>
       </c>
-      <c r="P29" s="33" t="s">
+      <c r="P29" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="Q29" s="33" t="s">
+      <c r="Q29" s="41" t="s">
         <v>73</v>
       </c>
-      <c r="R29" s="33" t="s">
+      <c r="R29" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="S29" s="38">
+      <c r="S29" s="39">
         <v>18.0</v>
       </c>
-      <c r="T29" s="55">
+      <c r="T29" s="58">
         <v>0.6666666666666666</v>
       </c>
-      <c r="U29" s="46" t="s">
+      <c r="U29" s="45" t="s">
         <v>74</v>
       </c>
-      <c r="V29" s="46" t="s">
+      <c r="V29" s="45" t="s">
         <v>69</v>
       </c>
-      <c r="W29" s="46" t="s">
+      <c r="W29" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="X29" s="54" t="s">
+      <c r="X29" s="57" t="s">
         <v>19</v>
       </c>
-      <c r="Y29" s="31">
+      <c r="Y29" s="49">
         <v>18.0</v>
       </c>
-      <c r="Z29" s="32">
+      <c r="Z29" s="50">
         <v>0.6666666666666666</v>
       </c>
-      <c r="AA29" s="46" t="s">
+      <c r="AA29" s="45" t="s">
         <v>75</v>
       </c>
-      <c r="AB29" s="46" t="s">
+      <c r="AB29" s="45" t="s">
         <v>21</v>
       </c>
-      <c r="AC29" s="46" t="s">
+      <c r="AC29" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="AD29" s="56" t="s">
+      <c r="AD29" s="59" t="s">
         <v>19</v>
       </c>
-      <c r="AE29" s="57"/>
-      <c r="AF29" s="58"/>
+      <c r="AE29" s="60"/>
+      <c r="AF29" s="61"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="31">
+      <c r="A30" s="49">
         <v>19.0</v>
       </c>
-      <c r="B30" s="32">
+      <c r="B30" s="50">
         <v>0.6805555555555556</v>
       </c>
-      <c r="C30" s="33" t="s">
+      <c r="C30" s="41" t="s">
         <v>76</v>
       </c>
-      <c r="D30" s="33" t="s">
+      <c r="D30" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="E30" s="33" t="s">
+      <c r="E30" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="F30" s="31"/>
-      <c r="G30" s="31">
+      <c r="F30" s="49"/>
+      <c r="G30" s="49">
         <v>19.0</v>
       </c>
-      <c r="H30" s="32">
+      <c r="H30" s="50">
         <v>0.6805555555555556</v>
       </c>
-      <c r="I30" s="33" t="s">
+      <c r="I30" s="41" t="s">
         <v>77</v>
       </c>
-      <c r="J30" s="33" t="s">
+      <c r="J30" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="K30" s="33" t="s">
+      <c r="K30" s="41" t="s">
         <v>63</v>
       </c>
-      <c r="L30" s="33" t="s">
+      <c r="L30" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="M30" s="31">
+      <c r="M30" s="49">
         <v>19.0</v>
       </c>
-      <c r="N30" s="32">
+      <c r="N30" s="50">
         <v>0.6805555555555556</v>
       </c>
-      <c r="O30" s="33" t="s">
+      <c r="O30" s="41" t="s">
         <v>78</v>
       </c>
-      <c r="P30" s="33" t="s">
+      <c r="P30" s="41" t="s">
         <v>69</v>
       </c>
-      <c r="Q30" s="33" t="s">
+      <c r="Q30" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="R30" s="33" t="s">
+      <c r="R30" s="41" t="s">
         <v>60</v>
       </c>
       <c r="S30" s="22">
@@ -2837,22 +2844,22 @@
       <c r="AF30" s="27"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="31">
+      <c r="A31" s="49">
         <v>20.0</v>
       </c>
-      <c r="B31" s="32">
+      <c r="B31" s="50">
         <v>0.6944444444444444</v>
       </c>
-      <c r="C31" s="33" t="s">
+      <c r="C31" s="41" t="s">
         <v>79</v>
       </c>
-      <c r="D31" s="33" t="s">
+      <c r="D31" s="41" t="s">
         <v>21</v>
       </c>
-      <c r="E31" s="33" t="s">
+      <c r="E31" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="F31" s="33" t="s">
+      <c r="F31" s="41" t="s">
         <v>16</v>
       </c>
       <c r="G31" s="22">
@@ -2865,18 +2872,18 @@
       <c r="J31" s="22"/>
       <c r="K31" s="22"/>
       <c r="L31" s="22"/>
-      <c r="M31" s="59">
+      <c r="M31" s="62">
         <v>20.0</v>
       </c>
-      <c r="N31" s="60">
+      <c r="N31" s="63">
         <v>0.6944444444444444</v>
       </c>
-      <c r="O31" s="61" t="s">
+      <c r="O31" s="64" t="s">
         <v>80</v>
       </c>
-      <c r="P31" s="62"/>
-      <c r="Q31" s="62"/>
-      <c r="R31" s="63"/>
+      <c r="P31" s="65"/>
+      <c r="Q31" s="65"/>
+      <c r="R31" s="66"/>
       <c r="S31" s="22">
         <v>20.0</v>
       </c>
@@ -2921,18 +2928,18 @@
       <c r="J32" s="22"/>
       <c r="K32" s="22"/>
       <c r="L32" s="22"/>
-      <c r="M32" s="59">
+      <c r="M32" s="62">
         <v>21.0</v>
       </c>
-      <c r="N32" s="60">
+      <c r="N32" s="63">
         <v>0.7083333333333334</v>
       </c>
-      <c r="O32" s="61" t="s">
+      <c r="O32" s="64" t="s">
         <v>80</v>
       </c>
-      <c r="P32" s="62"/>
-      <c r="Q32" s="62"/>
-      <c r="R32" s="63"/>
+      <c r="P32" s="65"/>
+      <c r="Q32" s="65"/>
+      <c r="R32" s="66"/>
       <c r="S32" s="22">
         <v>21.0</v>
       </c>
@@ -2977,18 +2984,18 @@
       <c r="J33" s="22"/>
       <c r="K33" s="22"/>
       <c r="L33" s="22"/>
-      <c r="M33" s="59">
+      <c r="M33" s="62">
         <v>22.0</v>
       </c>
-      <c r="N33" s="60">
+      <c r="N33" s="63">
         <v>0.7222222222222222</v>
       </c>
-      <c r="O33" s="61" t="s">
+      <c r="O33" s="64" t="s">
         <v>80</v>
       </c>
-      <c r="P33" s="62"/>
-      <c r="Q33" s="62"/>
-      <c r="R33" s="63"/>
+      <c r="P33" s="65"/>
+      <c r="Q33" s="65"/>
+      <c r="R33" s="66"/>
       <c r="S33" s="22">
         <v>22.0</v>
       </c>
@@ -3035,18 +3042,18 @@
       <c r="J34" s="22"/>
       <c r="K34" s="22"/>
       <c r="L34" s="22"/>
-      <c r="M34" s="59">
+      <c r="M34" s="62">
         <v>23.0</v>
       </c>
-      <c r="N34" s="60">
+      <c r="N34" s="63">
         <v>0.7361111111111112</v>
       </c>
-      <c r="O34" s="61" t="s">
+      <c r="O34" s="64" t="s">
         <v>80</v>
       </c>
-      <c r="P34" s="62"/>
-      <c r="Q34" s="62"/>
-      <c r="R34" s="63"/>
+      <c r="P34" s="65"/>
+      <c r="Q34" s="65"/>
+      <c r="R34" s="66"/>
       <c r="S34" s="22">
         <v>23.0</v>
       </c>
@@ -3091,18 +3098,18 @@
       <c r="J35" s="22"/>
       <c r="K35" s="22"/>
       <c r="L35" s="22"/>
-      <c r="M35" s="59">
+      <c r="M35" s="62">
         <v>24.0</v>
       </c>
-      <c r="N35" s="60">
+      <c r="N35" s="63">
         <v>0.75</v>
       </c>
-      <c r="O35" s="61" t="s">
+      <c r="O35" s="64" t="s">
         <v>80</v>
       </c>
-      <c r="P35" s="62"/>
-      <c r="Q35" s="62"/>
-      <c r="R35" s="63"/>
+      <c r="P35" s="65"/>
+      <c r="Q35" s="65"/>
+      <c r="R35" s="66"/>
       <c r="S35" s="22">
         <v>24.0</v>
       </c>
@@ -3147,18 +3154,18 @@
       <c r="J36" s="22"/>
       <c r="K36" s="22"/>
       <c r="L36" s="22"/>
-      <c r="M36" s="59">
+      <c r="M36" s="62">
         <v>25.0</v>
       </c>
-      <c r="N36" s="60">
+      <c r="N36" s="63">
         <v>0.7638888888888888</v>
       </c>
-      <c r="O36" s="61" t="s">
+      <c r="O36" s="64" t="s">
         <v>80</v>
       </c>
-      <c r="P36" s="62"/>
-      <c r="Q36" s="62"/>
-      <c r="R36" s="63"/>
+      <c r="P36" s="65"/>
+      <c r="Q36" s="65"/>
+      <c r="R36" s="66"/>
       <c r="S36" s="22">
         <v>25.0</v>
       </c>
@@ -3203,18 +3210,18 @@
       <c r="J37" s="22"/>
       <c r="K37" s="22"/>
       <c r="L37" s="22"/>
-      <c r="M37" s="59">
+      <c r="M37" s="62">
         <v>26.0</v>
       </c>
-      <c r="N37" s="60">
+      <c r="N37" s="63">
         <v>0.7777777777777778</v>
       </c>
-      <c r="O37" s="61" t="s">
+      <c r="O37" s="64" t="s">
         <v>80</v>
       </c>
-      <c r="P37" s="62"/>
-      <c r="Q37" s="62"/>
-      <c r="R37" s="63"/>
+      <c r="P37" s="65"/>
+      <c r="Q37" s="65"/>
+      <c r="R37" s="66"/>
       <c r="S37" s="22">
         <v>26.0</v>
       </c>
@@ -3259,18 +3266,18 @@
       <c r="J38" s="22"/>
       <c r="K38" s="22"/>
       <c r="L38" s="22"/>
-      <c r="M38" s="59">
+      <c r="M38" s="62">
         <v>27.0</v>
       </c>
-      <c r="N38" s="60">
+      <c r="N38" s="63">
         <v>0.7916666666666666</v>
       </c>
-      <c r="O38" s="61" t="s">
+      <c r="O38" s="64" t="s">
         <v>80</v>
       </c>
-      <c r="P38" s="62"/>
-      <c r="Q38" s="62"/>
-      <c r="R38" s="63"/>
+      <c r="P38" s="65"/>
+      <c r="Q38" s="65"/>
+      <c r="R38" s="66"/>
       <c r="S38" s="22">
         <v>27.0</v>
       </c>
@@ -3315,18 +3322,18 @@
       <c r="J39" s="22"/>
       <c r="K39" s="22"/>
       <c r="L39" s="22"/>
-      <c r="M39" s="59">
+      <c r="M39" s="62">
         <v>28.0</v>
       </c>
-      <c r="N39" s="60">
+      <c r="N39" s="63">
         <v>0.8055555555555556</v>
       </c>
-      <c r="O39" s="61" t="s">
+      <c r="O39" s="64" t="s">
         <v>80</v>
       </c>
-      <c r="P39" s="62"/>
-      <c r="Q39" s="62"/>
-      <c r="R39" s="63"/>
+      <c r="P39" s="65"/>
+      <c r="Q39" s="65"/>
+      <c r="R39" s="66"/>
       <c r="S39" s="22">
         <v>28.0</v>
       </c>
@@ -3346,7 +3353,7 @@
       <c r="AA39" s="22"/>
       <c r="AB39" s="22"/>
       <c r="AC39" s="22"/>
-      <c r="AD39" s="64"/>
+      <c r="AD39" s="67"/>
       <c r="AE39" s="1"/>
       <c r="AF39" s="1"/>
     </row>
@@ -3371,18 +3378,18 @@
       <c r="J40" s="22"/>
       <c r="K40" s="22"/>
       <c r="L40" s="22"/>
-      <c r="M40" s="59">
+      <c r="M40" s="62">
         <v>29.0</v>
       </c>
-      <c r="N40" s="60">
+      <c r="N40" s="63">
         <v>0.8194444444444444</v>
       </c>
-      <c r="O40" s="61" t="s">
+      <c r="O40" s="64" t="s">
         <v>80</v>
       </c>
-      <c r="P40" s="62"/>
-      <c r="Q40" s="62"/>
-      <c r="R40" s="63"/>
+      <c r="P40" s="65"/>
+      <c r="Q40" s="65"/>
+      <c r="R40" s="66"/>
       <c r="S40" s="22">
         <v>29.0</v>
       </c>
@@ -3402,7 +3409,7 @@
       <c r="AA40" s="22"/>
       <c r="AB40" s="22"/>
       <c r="AC40" s="22"/>
-      <c r="AD40" s="64"/>
+      <c r="AD40" s="67"/>
       <c r="AE40" s="1"/>
       <c r="AF40" s="1"/>
     </row>
@@ -3427,18 +3434,18 @@
       <c r="J41" s="22"/>
       <c r="K41" s="22"/>
       <c r="L41" s="22"/>
-      <c r="M41" s="59">
+      <c r="M41" s="62">
         <v>30.0</v>
       </c>
-      <c r="N41" s="60">
+      <c r="N41" s="63">
         <v>0.8333333333333334</v>
       </c>
-      <c r="O41" s="61" t="s">
+      <c r="O41" s="64" t="s">
         <v>80</v>
       </c>
-      <c r="P41" s="62"/>
-      <c r="Q41" s="62"/>
-      <c r="R41" s="63"/>
+      <c r="P41" s="65"/>
+      <c r="Q41" s="65"/>
+      <c r="R41" s="66"/>
       <c r="S41" s="22">
         <v>30.0</v>
       </c>
@@ -3458,7 +3465,7 @@
       <c r="AA41" s="22"/>
       <c r="AB41" s="22"/>
       <c r="AC41" s="22"/>
-      <c r="AD41" s="64"/>
+      <c r="AD41" s="67"/>
       <c r="AE41" s="1"/>
       <c r="AF41" s="1"/>
     </row>
@@ -3483,18 +3490,18 @@
       <c r="J42" s="22"/>
       <c r="K42" s="22"/>
       <c r="L42" s="22"/>
-      <c r="M42" s="59">
+      <c r="M42" s="62">
         <v>31.0</v>
       </c>
-      <c r="N42" s="60">
+      <c r="N42" s="63">
         <v>0.8472222222222222</v>
       </c>
-      <c r="O42" s="61" t="s">
+      <c r="O42" s="64" t="s">
         <v>80</v>
       </c>
-      <c r="P42" s="62"/>
-      <c r="Q42" s="62"/>
-      <c r="R42" s="63"/>
+      <c r="P42" s="65"/>
+      <c r="Q42" s="65"/>
+      <c r="R42" s="66"/>
       <c r="S42" s="22">
         <v>31.0</v>
       </c>
@@ -3514,63 +3521,63 @@
       <c r="AA42" s="22"/>
       <c r="AB42" s="22"/>
       <c r="AC42" s="22"/>
-      <c r="AD42" s="64"/>
+      <c r="AD42" s="67"/>
       <c r="AE42" s="1"/>
       <c r="AF42" s="1"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="65">
+      <c r="A43" s="68">
         <v>32.0</v>
       </c>
-      <c r="B43" s="66">
+      <c r="B43" s="69">
         <v>0.8611111111111112</v>
       </c>
-      <c r="C43" s="65"/>
-      <c r="D43" s="65"/>
-      <c r="E43" s="65"/>
-      <c r="F43" s="65"/>
-      <c r="G43" s="65">
+      <c r="C43" s="68"/>
+      <c r="D43" s="68"/>
+      <c r="E43" s="68"/>
+      <c r="F43" s="68"/>
+      <c r="G43" s="68">
         <v>32.0</v>
       </c>
-      <c r="H43" s="66">
+      <c r="H43" s="69">
         <v>0.8611111111111112</v>
       </c>
-      <c r="I43" s="65"/>
-      <c r="J43" s="65"/>
-      <c r="K43" s="65"/>
-      <c r="L43" s="65"/>
-      <c r="M43" s="67">
+      <c r="I43" s="68"/>
+      <c r="J43" s="68"/>
+      <c r="K43" s="68"/>
+      <c r="L43" s="68"/>
+      <c r="M43" s="70">
         <v>32.0</v>
       </c>
-      <c r="N43" s="68">
+      <c r="N43" s="71">
         <v>0.8611111111111112</v>
       </c>
-      <c r="O43" s="69" t="s">
+      <c r="O43" s="72" t="s">
         <v>80</v>
       </c>
-      <c r="P43" s="70"/>
-      <c r="Q43" s="70"/>
-      <c r="R43" s="71"/>
-      <c r="S43" s="65">
+      <c r="P43" s="73"/>
+      <c r="Q43" s="73"/>
+      <c r="R43" s="74"/>
+      <c r="S43" s="68">
         <v>32.0</v>
       </c>
-      <c r="T43" s="66">
+      <c r="T43" s="69">
         <v>0.8611111111111112</v>
       </c>
-      <c r="U43" s="65"/>
-      <c r="V43" s="65"/>
-      <c r="W43" s="65"/>
-      <c r="X43" s="65"/>
-      <c r="Y43" s="65">
+      <c r="U43" s="68"/>
+      <c r="V43" s="68"/>
+      <c r="W43" s="68"/>
+      <c r="X43" s="68"/>
+      <c r="Y43" s="68">
         <v>32.0</v>
       </c>
-      <c r="Z43" s="66">
+      <c r="Z43" s="69">
         <v>0.8611111111111112</v>
       </c>
-      <c r="AA43" s="65"/>
-      <c r="AB43" s="65"/>
-      <c r="AC43" s="65"/>
-      <c r="AD43" s="72"/>
+      <c r="AA43" s="68"/>
+      <c r="AB43" s="68"/>
+      <c r="AC43" s="68"/>
+      <c r="AD43" s="75"/>
       <c r="AE43" s="1"/>
       <c r="AF43" s="1"/>
     </row>

</xml_diff>